<commit_message>
Regenerate all outputs with dual-channel InnoHK search (ITC KPI)
</commit_message>
<xml_diff>
--- a/COCHE_Papers.xlsx
+++ b/COCHE_Papers.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COCHE Papers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'COCHE Papers'!$A$1:$I$266</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'COCHE Papers'!$A$1:$J$267</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I266"/>
+  <dimension ref="A1:J267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -468,8 +468,9 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,10 +511,15 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>All Authors</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -555,10 +561,15 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>Qiuqian Ou, Hongwei Chu, Yujian Liu, Liangling Cai, Zhenhe Huang, Dan Li, Jiating Lin, Yue Hu ...</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41378-026-01362-6</t>
         </is>
@@ -600,10 +611,15 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>Xingdao He, Matthew Chamberlin, Zhaoqi Chen, Jing Li, Yuyu Gao, Feng Guo, Yutao Ma, Xiaohe Wei ...</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.aee2752</t>
         </is>
@@ -645,10 +661,15 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>Bangul Khan, Rana Talha Khalid, Bilawal Khan, Muhammad Hasan Masrur, Mohamed Elhousseini Hilal, Mohamed Elgendi, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smll.74020</t>
         </is>
@@ -690,10 +711,15 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>Bolong Li, Kai Yang, Jinyu Shao, Zhihao Ma, Zhiheng Zeng, Dong Wang, Derek Ho</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d6mh00251j</t>
         </is>
@@ -735,10 +761,15 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
           <t>Hogi Hartanto, Jiaheng Li, Cheuk Chun Szeto, Ting-Hsuan Chen</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d6lc00249h</t>
         </is>
@@ -780,10 +811,15 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
           <t>Bangul Khan, Syed Bilal Ahmed, Bilawal Khan, Muhammad Shehzad Khan, Liangyi Lyu, Iyappan Gunasekaran, Rafi U Shan Ahmad, Junchen Liao ...</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d5tb02743h</t>
         </is>
@@ -825,10 +861,15 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
           <t>Xinran Chen, Xi Xu, Chongxue Bie, Peter van Zijl, Nirbhay Yadav, Jiadi Xu, Qizhi Yang, Tao Wang ...</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.70280</t>
         </is>
@@ -870,10 +911,15 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
           <t>Rafi U Shan Ahmad, Muhammad Shehzad Khan, Mohamed Elhousseini Hilal, Junchen Liao, Feng Chuhan, Wasim Ullah Khan, Bangul Khan, Mubasher Ali ...</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adhm.202505887</t>
         </is>
@@ -915,10 +961,15 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
           <t>Yue Hou, Qiong Liu, Zeru Wang, Xinru Yang, Dedi Li, Yiqiao Wang, Zhiquan Wei, Zhaodong Huang ...</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/jacs.5c23299</t>
         </is>
@@ -960,10 +1011,15 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
           <t>Ya Huang, Zhenlin Chen, Jingkun Zhou, Huiling Jia, Lung Chow, Yu Zhou, Shengxin Jia, Binbin Zhang ...</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.aed7673</t>
         </is>
@@ -1005,10 +1061,15 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
           <t>Zhiquan Wei, Jiaxiong Zhu, Yiqiao Wang, Xinru Yang, Dedi Li, Hong Hu, Qingshun Nian, Shaoce Zhang ...</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202524374</t>
         </is>
@@ -1050,10 +1111,15 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
           <t>Yang Liu, Zheng Qu, Yongchao Wang, Jingyi Zhu, Lidai Wang</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.ultras.2026.108095</t>
         </is>
@@ -1095,10 +1161,15 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
           <t>Bangul Khan, Bilawal Khan, Syed Bilal Ahmed, Wasim Ullah Khan, Junchen Liao, Md Shohidul Islam, Iyappan Gunasekaran, Rafi U Shan Ahmad ...</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smsc.202500526</t>
         </is>
@@ -1140,10 +1211,15 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
           <t>Lung Chow, Jianpeng Zhang, Zehua Peng, Denglin Ye, Binbin Zhang, Jian Li, Wooyoung Park, Chentao Du ...</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202524380</t>
         </is>
@@ -1185,10 +1261,15 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
           <t>Mingzi Liu, Jiahao Sun, Zuowei Sun, Yawen Xiao, Yi Chen, Jiyu Li, Xinge Yu</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d5lc00906e</t>
         </is>
@@ -1230,10 +1311,15 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
           <t>Youyang Wan, Xianglin Ji, Richard Yan-Do, Hailiang Sun, Chuanyin Xiong, Yongkang Zhang, Xi Zhao, Peilin Fang ...</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acssensors.5c03201</t>
         </is>
@@ -1275,10 +1361,15 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
           <t>Xiao Gu, Wei Tang, Jinpei Han, Veer Sangha, Fenglin Liu, Shreyank N Gowda, Antonio H Ribeiro, Patrick Schwab ...</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s42256-026-01180-5</t>
         </is>
@@ -1320,10 +1411,15 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
           <t>Yujie Pu, Peihua Dong, Lei He, Juan Huang, Yandi Wu, Jiang-Yun Luo, Qinghua Chen, Cheng-Lin Zhang ...</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1161/CIRCRESAHA.125.326815</t>
         </is>
@@ -1365,10 +1461,15 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
           <t>Mingze Sun, He Zhang, Xingdao He, Xi Wei, Binbin Cui, Hao Huang, Hao Li, Yuan Lin ...</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/nsr/nwag105</t>
         </is>
@@ -1410,10 +1511,15 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
           <t>Luyang Wang, James Chung Wai Cheung, Xia Zhao, Bee Luan Khoo, Siu Hong Dexter Wong</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/ijms27031330</t>
         </is>
@@ -1455,10 +1561,15 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
           <t>Chenyu Cui, Hogi Hartanto, Xinxue Yin, Jiaheng Li, Choi Wan Luk, Cheuk Chun Szeto, Ting-Hsuan Chen</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.bios.2026.118400</t>
         </is>
@@ -1500,10 +1611,15 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
           <t>Huabing Liu, Zilin Chen, Lok Hin Law, Yang Liu, Ziyan Wang, Jiawen Wang, Yi Zhang, Dinggang Shen ...</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s44172-025-00580-6</t>
         </is>
@@ -1545,10 +1661,15 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
           <t>Yiming Zhang, Shirong Qiu, Kai Du, Shun Wu, Ting Xiang, Kenghao Zheng, Zijun Liu, Hanjie Chen ...</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s40820-025-02003-9</t>
         </is>
@@ -1590,10 +1711,15 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
           <t>Jin Shi, Yanfang Li, Dingran Dong, Junyang Li, Tao Wen, Yue Tang, Qi Zhang, Fei Pan ...</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/molecules31010086</t>
         </is>
@@ -1635,10 +1761,15 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
           <t>Yuyu Gao, Jianpeng Zhang, Hehua Zhang, Lung Chow, Guangyao Zhao, Guihuan Guo, Chun Ki Yiu, Binbin Zhang ...</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1073/pnas.2520922122</t>
         </is>
@@ -1680,10 +1811,15 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
           <t>Hao Wang, Ho Ko, Thomas W Leung, Junzhe Huang, Junjie Sai, Yu Liang, Haipeng Li, Jie Zhang ...</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-66167-z</t>
         </is>
@@ -1725,10 +1861,15 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
           <t>Cunman Liang, Zhou Jiang, Shirong Qiu, Lei Zhao, Xinxin Mao, Xiao Yang, Yuanting Zhang, Ni Zhao</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-67118-4</t>
         </is>
@@ -1770,10 +1911,15 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
           <t>Huabing Liu, Ziyi Xia, Lok Hin Law, Zilin Chen, Jianpan Huang, Dinggang Shen, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.70159</t>
         </is>
@@ -1815,10 +1961,15 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
           <t>Dechao Zhang, Yuxuan Liu, Dedi Li, Shimei Li, Qi Xiong, Zhaodong Huang, Shixun Wang, Hu Hong ...</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202512960</t>
         </is>
@@ -1860,10 +2011,15 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
           <t>Qi Xiong, Ruijie Wang, Dedi Li, Ruhong Li, Shuoqing Zhang, Zhiquan Wei, Shimei Li, Dechao Zhang ...</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-65256-3</t>
         </is>
@@ -1905,10 +2061,15 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
           <t>Xinnian Yang, Jiayin Zhang, Yanli Song, Dengqiang Jia, Qingqi Hong, Yiqiang Zhan, Xiang Sean Zhou, Yining Dong ...</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-64940-8</t>
         </is>
@@ -1950,10 +2111,15 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
           <t>He Zhang, Weibin Jia, Mingze Sun, Yuxiang Chen, Xiaoyi Zhang, Hao Li, Xingdao He, Peng Shi ...</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.aea6883</t>
         </is>
@@ -1995,10 +2161,15 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
           <t>Zhiquan Wei, Ze Chen, Yiqiao Wang, Xinru Yang, Dedi Li, Zhuoxi Wu, Shaoce Zhang, Xintao Ma ...</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-65047-w</t>
         </is>
@@ -2040,10 +2211,15 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
           <t>Hongwei Chu, Wooyoung Park, Yue Hu, Zhenhe Huang, Rui Shi, Jiyu Li, Zhiyuan Li, Mengge Wu ...</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.5c12395</t>
         </is>
@@ -2085,10 +2261,15 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
           <t>Zhiquan Wei, Yiqiao Wang, Hu Hong, Ze Chen, Ao Chen, Shixun Wang, Shuo Yang, Yue Hou ...</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
+      <c r="J36" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-64344-8</t>
         </is>
@@ -2130,10 +2311,15 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
           <t>Jiadong Zhang, Yonghao Li, Zheren Li, Zhiming Cui, Pinxiong Li, Jun Li, Zhen Li, Yu Xie ...</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41551-025-01495-5</t>
         </is>
@@ -2175,10 +2361,15 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
           <t>Qi Zhang, Dong Sun</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202516592</t>
         </is>
@@ -2220,10 +2411,15 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
           <t>Ziyan Wang, Yingying Lin, Peng Cao, Pei Cai, Jiawen Wang, Huabin Zhang, Shihao Zeng, Chi Yan Lee ...</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/jmri.70147</t>
         </is>
@@ -2265,10 +2461,15 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
           <t>Yuanmeng Zhou, Weibin Jia, Jiexue Bi, Meng Liu, Liling Liu, Hang Zhou, Guofeng Gu, Zonggang Chen</t>
         </is>
       </c>
-      <c r="I40" s="3" t="inlineStr">
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.carbpol.2025.124372</t>
         </is>
@@ -2310,10 +2511,15 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
           <t>Bangul Khan, Umay Amara, Bilawal Khan, Wasim Ullah Khan, Rafi U Shan Ahmad, Muhammad Shehzad Khan, Mohamed Elhousseini Hilal, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I41" s="3" t="inlineStr">
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202507853</t>
         </is>
@@ -2355,10 +2561,15 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
           <t>Qi Xiong, Dedi Li, Shimei Li, Dechao Zhang, Ruhong Li, Shuoqing Zhang, Shixun Wang, Hu Hong ...</t>
         </is>
       </c>
-      <c r="I42" s="3" t="inlineStr">
+      <c r="J42" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adx5020</t>
         </is>
@@ -2400,10 +2611,15 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
           <t>Yutao Ma, Chuxiao Xiong, Feng Guo, Man Huang, Xi Xie, Qiongyu Guo, Peng Shi</t>
         </is>
       </c>
-      <c r="I43" s="3" t="inlineStr">
+      <c r="J43" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.biomaterials.2025.123721</t>
         </is>
@@ -2445,10 +2661,15 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
           <t>Xinru Yang, Zhiquan Wei, Honglu Hu, Hu Hong, Yiqiao Wang, Jiaxiong Zhu, Pei Li, Tairan Wang ...</t>
         </is>
       </c>
-      <c r="I44" s="3" t="inlineStr">
+      <c r="J44" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202510023</t>
         </is>
@@ -2490,10 +2711,15 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
           <t>Hu Hong, Zhiquan Wei, Yiqiao Wang, Xinru Yang, Xun Guo, Qingshun Nian, Xinliang Li, Qing Li ...</t>
         </is>
       </c>
-      <c r="I45" s="3" t="inlineStr">
+      <c r="J45" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1073/pnas.2511121122</t>
         </is>
@@ -2535,10 +2761,15 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
           <t>Xinxing Zhou, Yujie Lin, Bo Wu, Hujing Shu, Kerui Li, Qinghong Zhang, Yaogang Li, Chengyi Hou ...</t>
         </is>
       </c>
-      <c r="I46" s="3" t="inlineStr">
+      <c r="J46" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jcis.2025.138878</t>
         </is>
@@ -2580,10 +2811,15 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
           <t>Yang Liu, Se Weon Park, Lok Hin Law, Kexin Wang, Licheng Ju, Jiadi Xu, Kannie W Y Chan, Jianpan Huang</t>
         </is>
       </c>
-      <c r="I47" s="3" t="inlineStr">
+      <c r="J47" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/mrm.70048</t>
         </is>
@@ -2625,10 +2861,15 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
           <t>Yiming Liu, Xingcan Huang, Qiang Zhang, Wooyoung Park, Jinpei Wang, Jingyou Su, Zhao Zhao, Xue Wang ...</t>
         </is>
       </c>
-      <c r="I48" s="3" t="inlineStr">
+      <c r="J48" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.5c09857</t>
         </is>
@@ -2670,10 +2911,15 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
           <t>Jing Zhang, Yatian Fu, Ching Yin Fong, Haojun Hua, Wei Li, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I49" s="3" t="inlineStr">
+      <c r="J49" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d4lc00795f</t>
         </is>
@@ -2715,10 +2961,15 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
           <t>Wei Li, Jing Zhang, Junchen Liao, Mingze Zhu, Xinrui Wang, Xiang Zhou, Zhiqiang Ma, Mohamed Elhousseini Hilal ...</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
+      <c r="J50" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.analchem.5c00930</t>
         </is>
@@ -2760,10 +3011,15 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
           <t>Pikting Cheung, Wei Zhang, Muhammad Shehzad Khan, Irfan Ahmed, Yuanchao Liu, Fraser Hill, Xinyue Li, Condon Lau</t>
         </is>
       </c>
-      <c r="I51" s="3" t="inlineStr">
+      <c r="J51" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1080/01478885.2025.2523618</t>
         </is>
@@ -2805,10 +3061,15 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
           <t>Xingcan Huang, Qiang Zhang, Yawen Yang, Lung Chow, Jie Ma, Guoqiang Xu, Fang Guo, Xinxin He ...</t>
         </is>
       </c>
-      <c r="I52" s="3" t="inlineStr">
+      <c r="J52" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-61261-8</t>
         </is>
@@ -2850,10 +3111,15 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
           <t>Zhan Gao, Yang Fu, Qiang Zhang, Jian Li, Zhiyuan Li, Guihuan Guo, Dengfeng Li, Jingkun Zhou ...</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
+      <c r="J53" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41563-025-02268-w</t>
         </is>
@@ -2895,10 +3161,15 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
           <t>Xianrui Zhang, Zhen Liu, Xuan Luo, Yi Cao, Wencong Zhang, Honglin Li, Wei Li, Shuk Han Cheng ...</t>
         </is>
       </c>
-      <c r="I54" s="3" t="inlineStr">
+      <c r="J54" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.isci.2025.112868</t>
         </is>
@@ -2940,10 +3211,15 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
           <t>Rong Zhang, Xintao Ma, Shaoce Zhang, Huilin Cui, Chuan Li, Yanbo Wang, Qing Li, Chao Peng ...</t>
         </is>
       </c>
-      <c r="I55" s="3" t="inlineStr">
+      <c r="J55" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202507724</t>
         </is>
@@ -2985,10 +3261,15 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
           <t>Xiao Yang, Xiaonan Liu, Yeung Yeung Chau, Xuezhi Qin, Hong Zhu, Liang Peng, Kannie W Y Chan, Zuankai Wang</t>
         </is>
       </c>
-      <c r="I56" s="3" t="inlineStr">
+      <c r="J56" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d5sc01777g</t>
         </is>
@@ -3030,10 +3311,15 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
           <t>Mingyu Ye, Qing Yin, Qingmin Ji, Jiajia Deng, Hongbing Jia</t>
         </is>
       </c>
-      <c r="I57" s="3" t="inlineStr">
+      <c r="J57" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smll.202504209</t>
         </is>
@@ -3075,10 +3361,15 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
           <t>Yue Hou, Yiqiao Wang, Zhiquan Wei, Zhuoxi Wu, Dedi Li, Qing Li, Shimei Li, Ze Chen ...</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr">
+      <c r="J58" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202505147</t>
         </is>
@@ -3120,10 +3411,15 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
           <t>Wengang Liu, Ruili Liu, Lok Ting Chu, Xinlei Wang, Jianpeng Wu, Jiandong Ding, Ting Hsuan Chen</t>
         </is>
       </c>
-      <c r="I59" s="3" t="inlineStr">
+      <c r="J59" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/rb/rbaf043</t>
         </is>
@@ -3165,10 +3461,15 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
           <t>Shimei Li, Hu Hong, Xinru Yang, Dedi Li, Qi Xiong, Dechao Zhang, Shixun Wang, Zhaodong Huang ...</t>
         </is>
       </c>
-      <c r="I60" s="3" t="inlineStr">
+      <c r="J60" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202504333</t>
         </is>
@@ -3210,10 +3511,15 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
           <t>Ke Huang, Zhiqiang Ma, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I61" s="3" t="inlineStr">
+      <c r="J61" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202415215</t>
         </is>
@@ -3255,10 +3561,15 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
           <t>Irfan Ahmed, Muhammad Shehzad Khan, Pikting Cheung, Hina Magsi, Zulfiqar Ali, Yanpeng Zhang, Martin Alda, Veerle Bergink ...</t>
         </is>
       </c>
-      <c r="I62" s="3" t="inlineStr">
+      <c r="J62" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jtemb.2025.127653</t>
         </is>
@@ -3300,10 +3611,15 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
           <t>Yanbo Wang, Yeyang Jia, Chuan Li, Huilin Cui, Rong Zhang, Hu Hong, Qing Li, Donghong Wang ...</t>
         </is>
       </c>
-      <c r="I63" s="3" t="inlineStr">
+      <c r="J63" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smtd.202500031</t>
         </is>
@@ -3345,10 +3661,15 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
           <t>Wei Li, Xinrui Wang, Mingze Zhu, Xin Huang, Pacifique Hirwa Umutoni, Ting-Hsuan Chen, Jian Lu, Shih-Chi Chen ...</t>
         </is>
       </c>
-      <c r="I64" s="3" t="inlineStr">
+      <c r="J64" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.talanta.2025.128100</t>
         </is>
@@ -3390,10 +3711,15 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
           <t>Chunki Yiu, Yiming Liu, Wooyoung Park, Jian Li, Xingcan Huang, Kuanming Yao, Yuyu Gao, Guangyao Zhao ...</t>
         </is>
       </c>
-      <c r="I65" s="3" t="inlineStr">
+      <c r="J65" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adt6041</t>
         </is>
@@ -3435,10 +3761,15 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
           <t>Yanbo Wang, Xintao Ma, Xinru Yang, Rong Zhang, Hu Hong, Shixun Wang, Qing Li, Ze Chen ...</t>
         </is>
       </c>
-      <c r="I66" s="3" t="inlineStr">
+      <c r="J66" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202419702</t>
         </is>
@@ -3480,10 +3811,15 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
           <t>Guoqiang Xu, Haoyu Wang, Guangyao Zhao, Jingjing Fu, Kuanming Yao, Shengxin Jia, Rui Shi, Xingcan Huang ...</t>
         </is>
       </c>
-      <c r="I67" s="3" t="inlineStr">
+      <c r="J67" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adt0318</t>
         </is>
@@ -3525,10 +3861,15 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
           <t>Qiuna Zhuang, Kuanming Yao, Xian Song, Qiang Zhang, Chi Zhang, Huiming Wang, Ruofan Yang, Guangyao Zhao ...</t>
         </is>
       </c>
-      <c r="I68" s="3" t="inlineStr">
+      <c r="J68" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adu3146</t>
         </is>
@@ -3570,10 +3911,15 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
           <t>Han Zhang, Qiguang Chen, Lok Ming Lui</t>
         </is>
       </c>
-      <c r="I69" s="3" t="inlineStr">
+      <c r="J69" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.neunet.2025.107378</t>
         </is>
@@ -3615,10 +3961,15 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
           <t>Rafi U Shan Ahmad, Wasim Ullah Khan, Muhammad Shehzad Khan, Pikting Cheung</t>
         </is>
       </c>
-      <c r="I70" s="3" t="inlineStr">
+      <c r="J70" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.mtbio.2025.101663</t>
         </is>
@@ -3660,10 +4011,15 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
           <t>Zhibiao Tian, Yatian Fu, Zhiyong Dang, Tao Guo, Wenjuan Li, Jing Zhang</t>
         </is>
       </c>
-      <c r="I71" s="3" t="inlineStr">
+      <c r="J71" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/nano15060434</t>
         </is>
@@ -3705,10 +4061,15 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
           <t>Shixun Wang, Shengnan Wang, Zhiquan Wei, Yiqiao Wang, Dechao Zhang, Ze Chen, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I72" s="3" t="inlineStr">
+      <c r="J72" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-025-56607-1</t>
         </is>
@@ -3750,10 +4111,15 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
           <t>Weijie Wu, Wenhai Sui, Sizhe Chen, Ziheng Guo, Xu Jing, Xiaolu Wang, Qun Wang, Xinshuang Yu ...</t>
         </is>
       </c>
-      <c r="I73" s="3" t="inlineStr">
+      <c r="J73" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cmet.2025.01.006</t>
         </is>
@@ -3795,10 +4161,15 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
           <t>Zhiqiang Ma, Jing Zhang, Shangjie Zou, Ke Huang, Wei Li, Mohamed Elhousseini Hilal, Mingze Zhu, Yatian Fu ...</t>
         </is>
       </c>
-      <c r="I74" s="3" t="inlineStr">
+      <c r="J74" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.4c09980</t>
         </is>
@@ -3840,10 +4211,15 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
           <t>Shixun Wang, Zhiquan Wei, Hu Hong, Xun Guo, Yiqiao Wang, Ze Chen, Dechao Zhang, Xiaoyu Zhang ...</t>
         </is>
       </c>
-      <c r="I75" s="3" t="inlineStr">
+      <c r="J75" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-55385-6</t>
         </is>
@@ -3885,10 +4261,15 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
           <t>Tianyi Dai, Yankun Lin, Qing Yin, Qingmin Ji, Jingyi Wang, Hongbing Jia</t>
         </is>
       </c>
-      <c r="I76" s="3" t="inlineStr">
+      <c r="J76" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jcis.2025.01.031</t>
         </is>
@@ -3930,10 +4311,15 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
           <t>Xinliang Li, Tong Liu, Pei Li, Guojin Liang, Zhaodong Huang, Ze Chen, Ao Chen, Yuefeng Su ...</t>
         </is>
       </c>
-      <c r="I77" s="3" t="inlineStr">
+      <c r="J77" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.4c16550</t>
         </is>
@@ -3975,10 +4361,15 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
           <t>Jing Zhang, Wei Qiao, Rui Jin, Hongjin Li, Hui Gong, Shih-Chi Chen, Qingming Luo, Jing Yuan</t>
         </is>
       </c>
-      <c r="I78" s="3" t="inlineStr">
+      <c r="J78" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41377-024-01677-x</t>
         </is>
@@ -4020,10 +4411,15 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
           <t>Wasim Ullah Khan, Mohammed Alissa, Khaled S Allemailem, Faris Alrumaihi, Hajed Obaid Alharbi, Nahlah Makki Almansour, Leen A Aldaiji, Marwh Jamal Albalawi ...</t>
         </is>
       </c>
-      <c r="I79" s="3" t="inlineStr">
+      <c r="J79" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cpcardiol.2024.102964</t>
         </is>
@@ -4065,10 +4461,15 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
           <t>Shimei Li, Hu Hong, Dedi Li, Xinru Yang, Shixun Wang, Dechao Zhang, Qi Xiong, Zhaodong Huang ...</t>
         </is>
       </c>
-      <c r="I80" s="3" t="inlineStr">
+      <c r="J80" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202409500</t>
         </is>
@@ -4110,10 +4511,15 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
           <t>Haoyun Su, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I81" s="3" t="inlineStr">
+      <c r="J81" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.4c05923</t>
         </is>
@@ -4155,10 +4561,15 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
           <t>Aqiang Liu, Zheng Zhang, Jing Li, Hui Yu, Nana Wang, Jianpu Wang, Ni Zhao</t>
         </is>
       </c>
-      <c r="I82" s="3" t="inlineStr">
+      <c r="J82" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202414788</t>
         </is>
@@ -4200,10 +4611,15 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
           <t>Lung Chow, Qiang Zhang, Xingcan Huang, Jun Zhang, Jingkun Zhou, Bo Zhu, Jiyu Li, Ya Huang ...</t>
         </is>
       </c>
-      <c r="I83" s="3" t="inlineStr">
+      <c r="J83" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202406798</t>
         </is>
@@ -4245,10 +4661,15 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
           <t>Hong Zhu, Jinpei Wang, Xiao Yang, Baoping Zhang, Zuankai Wang</t>
         </is>
       </c>
-      <c r="I84" s="3" t="inlineStr">
+      <c r="J84" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202413112</t>
         </is>
@@ -4290,10 +4711,15 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
           <t>Yixue Duan, Bolong Li, Kai Yang, Zheng Gong, Xuqiao Peng, Liang He, Derek Ho</t>
         </is>
       </c>
-      <c r="I85" s="3" t="inlineStr">
+      <c r="J85" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s40820-024-01586-z</t>
         </is>
@@ -4335,10 +4761,15 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
           <t>Kai Yang, Bolong Li, Zhihao Ma, Jiangang Xu, Dong Wang, Zhiheng Zeng, Derek Ho</t>
         </is>
       </c>
-      <c r="I86" s="3" t="inlineStr">
+      <c r="J86" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202415000</t>
         </is>
@@ -4380,10 +4811,15 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
           <t>Shimei Li, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I87" s="3" t="inlineStr">
+      <c r="J87" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202413515</t>
         </is>
@@ -4425,10 +4861,15 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
           <t>Jin Qu, Yuan Wang, Chuxiao Xiong, Mingxue Wang, Xingdao He, Weibin Jia, Cheuk Yin Li, Tianlong Zhang ...</t>
         </is>
       </c>
-      <c r="I88" s="3" t="inlineStr">
+      <c r="J88" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-54292-0</t>
         </is>
@@ -4470,10 +4911,15 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
           <t>Yiming Liu, Wooyoung Park, Chun Ki Yiu, Xingcan Huang, Shengxin Jia, Yao Chen, Hehua Zhang, Hongting Chen ...</t>
         </is>
       </c>
-      <c r="I89" s="3" t="inlineStr">
+      <c r="J89" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1073/pnas.2412116121</t>
         </is>
@@ -4515,10 +4961,15 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
           <t>Jin Qu, Kai Xie, Shu Chen, Xingdao He, Yuan Wang, Matthew Chamberlin, Xi Zhao, Guangyu Zhu ...</t>
         </is>
       </c>
-      <c r="I90" s="3" t="inlineStr">
+      <c r="J90" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adq9207</t>
         </is>
@@ -4560,10 +5011,15 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
           <t>Feng Guo, Xianglin Ji, Chuxiao Xiong, Hailiang Sun, Zhenghua Liang, Richard Yan-Do, Baowen Gai, Feng Gao ...</t>
         </is>
       </c>
-      <c r="I91" s="3" t="inlineStr">
+      <c r="J91" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-53419-7</t>
         </is>
@@ -4605,10 +5061,15 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Zhaodong Huang, Chenlu Wang, Dedi Li, Qi Xiong, Yanbo Wang, Yue Hou, Yanlei Wang ...</t>
         </is>
       </c>
-      <c r="I92" s="3" t="inlineStr">
+      <c r="J92" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202406683</t>
         </is>
@@ -4650,10 +5111,15 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
           <t>Jingkun Zhou, Jian Li, Huiling Jia, Kuanming Yao, Shengxin Jia, Jiyu Li, Guangyao Zhao, Chun Ki Yiu ...</t>
         </is>
       </c>
-      <c r="I93" s="3" t="inlineStr">
+      <c r="J93" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-54249-3</t>
         </is>
@@ -4695,10 +5161,15 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
           <t>Zhiquan Wei, Guangmeng Qu, Zhaodong Huang, Yiqiao Wang, Dedi Li, Xinru Yang, Shaoce Zhang, Ao Chen ...</t>
         </is>
       </c>
-      <c r="I94" s="3" t="inlineStr">
+      <c r="J94" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202414388</t>
         </is>
@@ -4740,10 +5211,15 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
           <t>Jiangang Xu, Qiang Li, Derek Ho</t>
         </is>
       </c>
-      <c r="I95" s="3" t="inlineStr">
+      <c r="J95" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d4mh01067a</t>
         </is>
@@ -4785,10 +5261,15 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
           <t>Umay Amara, Lingtian Xu, Iftikhar Hussain, Kai Yang, Haibo Hu, Derek Ho</t>
         </is>
       </c>
-      <c r="I96" s="3" t="inlineStr">
+      <c r="J96" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smll.202405047</t>
         </is>
@@ -4830,10 +5311,15 @@
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
           <t>Vivian W M Leung, Se Weon Park, Joseph H C Lai, Zilin Chen, Jianpan Huang, Yang Liu, Charles Hu, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I97" s="3" t="inlineStr">
+      <c r="J97" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/mrm.30362</t>
         </is>
@@ -4875,10 +5361,15 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
           <t>Jun Ma, Yao Zhang, Song Gu, Cheng Ge, Shihao Mae, Adamo Young, Cheng Zhu, Xin Yang ...</t>
         </is>
       </c>
-      <c r="I98" s="3" t="inlineStr">
+      <c r="J98" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S2589-7500(24)00154-7</t>
         </is>
@@ -4920,10 +5411,15 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
           <t>Russell W Chan, Giles Hamilton-Fletcher, Bradley J Edelman, Muneeb A Faiq, Thajunnisa A Sajitha, Steen Moeller, Kevin C Chan</t>
         </is>
       </c>
-      <c r="I99" s="3" t="inlineStr">
+      <c r="J99" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1162/imag_a_00325</t>
         </is>
@@ -4965,10 +5461,15 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
           <t>Guihuan Guo, Chenyu Cui, Hogi Hartanto, Jiaheng Li, Ting-Hsuan Chen</t>
         </is>
       </c>
-      <c r="I100" s="3" t="inlineStr">
+      <c r="J100" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.talanta.2024.127089</t>
         </is>
@@ -5010,10 +5511,15 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
           <t>Kuanming Yao, Qiuna Zhuang, Qiang Zhang, Jingkun Zhou, Chun Ki Yiu, Jianpeng Zhang, Denglin Ye, Yawen Yang ...</t>
         </is>
       </c>
-      <c r="I101" s="3" t="inlineStr">
+      <c r="J101" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adq9575</t>
         </is>
@@ -5055,10 +5561,15 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
           <t>Shaoce Zhang, Hu Hong, Rong Zhang, Zhiquan Wei, Yiqiao Wang, Dong Chen, Chuan Li, Pei Li ...</t>
         </is>
       </c>
-      <c r="I102" s="3" t="inlineStr">
+      <c r="J102" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202412830</t>
         </is>
@@ -5100,10 +5611,15 @@
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
           <t>Hu Hong, Yu Wang, Yaqin Zhang, Bing Han, Qing Li, Xun Guo, Ying Guo, Ao Chen ...</t>
         </is>
       </c>
-      <c r="I103" s="3" t="inlineStr">
+      <c r="J103" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202407150</t>
         </is>
@@ -5145,10 +5661,15 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
           <t>Fei Pan, Yutong Wu, Kangning Cui, Shuxun Chen, Yanfang Li, Yaofang Liu, Adnan Shakoor, Han Zhao ...</t>
         </is>
       </c>
-      <c r="I104" s="3" t="inlineStr">
+      <c r="J104" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.compbiomed.2024.109151</t>
         </is>
@@ -5190,10 +5711,15 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
           <t>Hu Hong, Yiqiao Wang, Zhiquan Wei, Xinru Yang, Zhuoxi Wu, Xun Guo, Ao Chen, Shaoce Zhang ...</t>
         </is>
       </c>
-      <c r="I105" s="3" t="inlineStr">
+      <c r="J105" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202410209</t>
         </is>
@@ -5235,10 +5761,15 @@
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Jiaxiong Zhu, Shuo Yang, Zhiquan Wei, Yiqiao Wang, Ao Chen, Zhaodong Huang, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I106" s="3" t="inlineStr">
+      <c r="J106" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202411443</t>
         </is>
@@ -5280,10 +5811,15 @@
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
           <t>Chongyun Wang, Wah Shing Lam, Hanjin Huang, Han Zhao, Chunqi Zhang, Dong Sun</t>
         </is>
       </c>
-      <c r="I107" s="3" t="inlineStr">
+      <c r="J107" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1364/BOE.535028</t>
         </is>
@@ -5325,10 +5861,15 @@
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
           <t>Jian Li, Shengxin Jia, Dengfeng Li, Lung Chow, Qiang Zhang, Yiyuan Yang, Xiao Bai, Qingao Qu ...</t>
         </is>
       </c>
-      <c r="I108" s="3" t="inlineStr">
+      <c r="J108" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-51987-2</t>
         </is>
@@ -5370,10 +5911,15 @@
       </c>
       <c r="H109" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
           <t>Weibin Jia, Runrun Li, Fengjuan Zou, Min Li, Hongjuan Weng, Qianqian Shen, Guozhen Qi, Ruipiao Zhou ...</t>
         </is>
       </c>
-      <c r="I109" s="3" t="inlineStr">
+      <c r="J109" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adhm.202402158</t>
         </is>
@@ -5415,10 +5961,15 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
           <t>Yang Sylvia Liu, Chengqian Zhang, Bee Luan Khoo, Piliang Hao, Song Lin Chua</t>
         </is>
       </c>
-      <c r="I110" s="3" t="inlineStr">
+      <c r="J110" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jare.2024.08.038</t>
         </is>
@@ -5460,10 +6011,15 @@
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
           <t>Feifei Shi, Yudong Wu, Binyan Wang, Jiawei Bai, Yihan Ren, Tao Yang, Funian Mo, Derek Ho ...</t>
         </is>
       </c>
-      <c r="I111" s="3" t="inlineStr">
+      <c r="J111" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d4sc04851b</t>
         </is>
@@ -5505,10 +6061,15 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
           <t>Haoyun Su, Lok Hin Law, Yang Liu, Jianpan Huang, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I112" s="3" t="inlineStr">
+      <c r="J112" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.5238</t>
         </is>
@@ -5550,10 +6111,15 @@
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
           <t>Yoyo Wing Suet Yeung, Yeping Ma, Yanlin Deng, Bee Luan Khoo, Song Lin Chua</t>
         </is>
       </c>
-      <c r="I113" s="3" t="inlineStr">
+      <c r="J113" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202404467</t>
         </is>
@@ -5595,10 +6161,15 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
           <t>Kewang Nan, Kiwan Wong, Dengfeng Li, Binbin Ying, James C McRae, Vivian R Feig, Shubing Wang, Ningjie Du ...</t>
         </is>
       </c>
-      <c r="I114" s="3" t="inlineStr">
+      <c r="J114" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-51102-5</t>
         </is>
@@ -5640,10 +6211,15 @@
       </c>
       <c r="H115" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
           <t>Hrisheekesh Thachoth Chandran, Ruijie Ma, Zhihan Xu, Jipsa Chelora Veetil, Yongmin Luo, Top Archie Dela Peña, Iyappan Gunasekaran, Sudhi Mahadevan ...</t>
         </is>
       </c>
-      <c r="I115" s="3" t="inlineStr">
+      <c r="J115" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202407271</t>
         </is>
@@ -5685,10 +6261,15 @@
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
           <t>Qiang Zhang, Guangyao Zhao, Zhiyuan Li, Fang Guo, Ya Huang, Guihuan Guo, Jiachen Wang, Jingkun Zhou ...</t>
         </is>
       </c>
-      <c r="I116" s="3" t="inlineStr">
+      <c r="J116" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.bios.2024.116597</t>
         </is>
@@ -5730,10 +6311,15 @@
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
           <t>Deyuan Yang, Cheng Li, Yutong Kong, Yian Pei, Bing Miao, Gaole Dai, Pi Ding, Peng Shi ...</t>
         </is>
       </c>
-      <c r="I117" s="3" t="inlineStr">
+      <c r="J117" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/jacs.4c05205</t>
         </is>
@@ -5775,10 +6361,15 @@
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
           <t>Hui Li, Kai Yang, Haibo Hu, Chengbing Qin, Benli Yu, Sheng Zhou, Tongtong Jiang, Derek Ho</t>
         </is>
       </c>
-      <c r="I118" s="3" t="inlineStr">
+      <c r="J118" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.analchem.4c01484</t>
         </is>
@@ -5820,10 +6411,15 @@
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
           <t>Senlin Hou, Qingyun Huang, Hongyu Zhang, Qingjiu Chen, Cong Wu, Mengge Wu, Chen Meng, Kuanming Yao ...</t>
         </is>
       </c>
-      <c r="I119" s="3" t="inlineStr">
+      <c r="J119" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202400234</t>
         </is>
@@ -5865,10 +6461,15 @@
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
           <t>Chenyu Cui, Guihuan Guo, Ting-Hsuan Chen</t>
         </is>
       </c>
-      <c r="I120" s="3" t="inlineStr">
+      <c r="J120" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/biot.202400097</t>
         </is>
@@ -5910,10 +6511,15 @@
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
           <t>Jiahui He, Mengjia Zheng, Tianli Hu, Ya Huang, Jingyou Su, Chunyi Zhi, Xinge Yu, Chenjie Xu</t>
         </is>
       </c>
-      <c r="I121" s="3" t="inlineStr">
+      <c r="J121" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.34133/bmef.0044</t>
         </is>
@@ -5955,10 +6561,15 @@
       </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
           <t>Jian Li, Hongwei Chu, Zhenlin Chen, Chun Ki Yiu, Qing'ao Qu, Zhiyuan Li, Xinge Yu</t>
         </is>
       </c>
-      <c r="I122" s="3" t="inlineStr">
+      <c r="J122" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.4c04291</t>
         </is>
@@ -6000,10 +6611,15 @@
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
           <t>Shixun Wang, Zhaodong Huang, Jiaxiong Zhu, Yiqiao Wang, Dedi Li, Zhiquan Wei, Hu Hong, Dechao Zhang ...</t>
         </is>
       </c>
-      <c r="I123" s="3" t="inlineStr">
+      <c r="J123" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202406451</t>
         </is>
@@ -6045,10 +6661,15 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I124" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Zhaodong Huang, Jiaxiong Zhu, Dedi Li, Ao Chen, Zhiquan Wei, Yiqiao Wang, Nan Li ...</t>
         </is>
       </c>
-      <c r="I124" s="3" t="inlineStr">
+      <c r="J124" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202402898</t>
         </is>
@@ -6090,10 +6711,15 @@
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
           <t>Xinliang Li, Yanlei Wang, Junfeng Lu, Pei Li, Zhaodong Huang, Guojin Liang, Hongyan He, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I125" s="3" t="inlineStr">
+      <c r="J125" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adl0587</t>
         </is>
@@ -6135,10 +6761,15 @@
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I126" s="3" t="inlineStr">
+        <is>
           <t>Rong Zhang, Yaqin Zhang, Bo Xiao, Shaoce Zhang, Yanbo Wang, Huilin Cui, Chuan Li, Yue Hou ...</t>
         </is>
       </c>
-      <c r="I126" s="3" t="inlineStr">
+      <c r="J126" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202407589</t>
         </is>
@@ -6180,10 +6811,15 @@
       </c>
       <c r="H127" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
           <t>Yuan Wang, Jin Qu, Chuxiao Xiong, Bing Chen, Kai Xie, Mingxue Wang, Zhen Liu, Zhao Yue ...</t>
         </is>
       </c>
-      <c r="I127" s="3" t="inlineStr">
+      <c r="J127" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1073/pnas.2322264121</t>
         </is>
@@ -6225,10 +6861,15 @@
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I128" s="3" t="inlineStr">
+        <is>
           <t>Zilin Chen, Yekkuni L Balachandran, Wai Po Chong, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I128" s="3" t="inlineStr">
+      <c r="J128" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/ijms25115803</t>
         </is>
@@ -6270,10 +6911,15 @@
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
           <t>Dechao Zhang, Yuxuan Liu, Shuo Yang, Jiaxiong Zhu, Hu Hong, Shimei Li, Qi Xiong, Zhaodong Huang ...</t>
         </is>
       </c>
-      <c r="I129" s="3" t="inlineStr">
+      <c r="J129" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202401549</t>
         </is>
@@ -6315,10 +6961,15 @@
       </c>
       <c r="H130" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I130" s="3" t="inlineStr">
+        <is>
           <t>Yiming Liu, Shengxin Jia, Chun Ki Yiu, Wooyoung Park, Zhenlin Chen, Jin Nan, Xingcan Huang, Hongting Chen ...</t>
         </is>
       </c>
-      <c r="I130" s="3" t="inlineStr">
+      <c r="J130" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-48884-z</t>
         </is>
@@ -6360,10 +7011,15 @@
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="inlineStr">
+        <is>
           <t>Zhen Liu, Xuan Luo, Richard Yan-Do, Yuan Wang, Xi Xie, Zhongping Li, Shuk Han Cheng, Peng Shi</t>
         </is>
       </c>
-      <c r="I131" s="3" t="inlineStr">
+      <c r="J131" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acschemneuro.4c00158</t>
         </is>
@@ -6405,10 +7061,15 @@
       </c>
       <c r="H132" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I132" s="3" t="inlineStr">
+        <is>
           <t>Jiaheng Li, Lok Ting Chu, Hogi Hartanto, Guihuan Guo, Lu Liu, Jianpeng Wu, Minghui Wu, Chenyu Cui ...</t>
         </is>
       </c>
-      <c r="I132" s="3" t="inlineStr">
+      <c r="J132" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d4lc00118d</t>
         </is>
@@ -6450,10 +7111,15 @@
       </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
           <t>Zhiquan Wei, Zhaodong Huang, Guojin Liang, Yiqiao Wang, Shixun Wang, Yihan Yang, Tao Hu, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I133" s="3" t="inlineStr">
+      <c r="J133" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-48263-8</t>
         </is>
@@ -6495,10 +7161,15 @@
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I134" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Tairan Wang, Zhuoxi Wu, Yue Hou, Ao Chen, Yanbo Wang, Zhaodong Huang, Oliver G Schmidt ...</t>
         </is>
       </c>
-      <c r="I134" s="3" t="inlineStr">
+      <c r="J134" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-47950-w</t>
         </is>
@@ -6540,10 +7211,15 @@
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I135" s="3" t="inlineStr">
+        <is>
           <t>Zhenlin Chen, Lei Fan, Shuxun Chen, Han Zhao, Qiang Zhang, Yun Qu, Ya Huang, Xinge Yu ...</t>
         </is>
       </c>
-      <c r="I135" s="3" t="inlineStr">
+      <c r="J135" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adhm.202304532</t>
         </is>
@@ -6585,10 +7261,15 @@
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I136" s="3" t="inlineStr">
+        <is>
           <t>Shixun Wang, Yiqiao Wang, Zhiquan Wei, Jiaxiong Zhu, Ze Chen, Hu Hong, Qi Xiong, Dechao Zhang ...</t>
         </is>
       </c>
-      <c r="I136" s="3" t="inlineStr">
+      <c r="J136" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202401924</t>
         </is>
@@ -6630,10 +7311,15 @@
       </c>
       <c r="H137" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
           <t>Qing Li, Nan Li, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I137" s="3" t="inlineStr">
+      <c r="J137" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.nanolett.4c00101</t>
         </is>
@@ -6675,10 +7361,15 @@
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I138" s="3" t="inlineStr">
+        <is>
           <t>Binbin Zhang, Jiyu Li, Jingkun Zhou, Lung Chow, Guangyao Zhao, Ya Huang, Zhiqiang Ma, Qiang Zhang ...</t>
         </is>
       </c>
-      <c r="I138" s="3" t="inlineStr">
+      <c r="J138" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41586-024-07161-1</t>
         </is>
@@ -6720,10 +7411,15 @@
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I139" s="3" t="inlineStr">
+        <is>
           <t>Rohith Saai Pemmasani Prabakaran, Se Weon Park, Joseph H C Lai, Kexin Wang, Jiadi Xu, Zilin Chen, Abdul-Mojeed Olabisi Ilyas, Huabing Liu ...</t>
         </is>
       </c>
-      <c r="I139" s="3" t="inlineStr">
+      <c r="J139" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.5130</t>
         </is>
@@ -6765,10 +7461,15 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I140" s="3" t="inlineStr">
+        <is>
           <t>Yuanmeng Zhou, Weibin Jia, Jiexue Bi, Meng Liu, Liling Liu, Hang Zhou, Guofeng Gu, Zonggang Chen</t>
         </is>
       </c>
-      <c r="I140" s="3" t="inlineStr">
+      <c r="J140" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.carbpol.2024.122025</t>
         </is>
@@ -6810,10 +7511,15 @@
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I141" s="3" t="inlineStr">
+        <is>
           <t>Gaobo Wang, Yuyue Zhang, Hoi Kwan Kwong, Mengjia Zheng, Jianpeng Wu, Chenyu Cui, Kannie W Y Chan, Chenjie Xu ...</t>
         </is>
       </c>
-      <c r="I141" s="3" t="inlineStr">
+      <c r="J141" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202306188</t>
         </is>
@@ -6855,10 +7561,15 @@
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I142" s="3" t="inlineStr">
+        <is>
           <t>Hongzhen Liu, Xianglin Ji, Zihao Guo, Xi Wei, Jinchen Fan, Peng Shi, Xiong Pu, Feng Gong ...</t>
         </is>
       </c>
-      <c r="I142" s="3" t="inlineStr">
+      <c r="J142" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-024-45931-7</t>
         </is>
@@ -6900,10 +7611,15 @@
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="inlineStr">
+        <is>
           <t>Yulong Gao, Jimin Fu, Funian Mo, Lixin Zhang, Derek Ho, Haibo Hu</t>
         </is>
       </c>
-      <c r="I143" s="3" t="inlineStr">
+      <c r="J143" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smll.202400085</t>
         </is>
@@ -6945,10 +7661,15 @@
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I144" s="3" t="inlineStr">
+        <is>
           <t>Haojun Hua, Yanlin Deng, Jing Zhang, Xiang Zhou, Tianfu Zhang, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I144" s="3" t="inlineStr">
+      <c r="J144" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.bios.2024.116086</t>
         </is>
@@ -6990,10 +7711,15 @@
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I145" s="3" t="inlineStr">
+        <is>
           <t>Shengmei Chen, Shimei Li, Longtao Ma, Yiran Ying, Zhuoxi Wu, Haitao Huang, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I145" s="3" t="inlineStr">
+      <c r="J145" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202319125</t>
         </is>
@@ -7035,10 +7761,15 @@
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I146" s="3" t="inlineStr">
+        <is>
           <t>Jianpan Huang, Zilin Chen, Peter C M van Zijl, Lok Hin Law, Rohith Saai Pemmasani Prabakaran, Se Weon Park, Jiadi Xu, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I146" s="3" t="inlineStr">
+      <c r="J146" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/mrm.30035</t>
         </is>
@@ -7080,10 +7811,15 @@
       </c>
       <c r="H147" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="inlineStr">
+        <is>
           <t>Yeping Ma, Wing Suet Tang, Sylvia Yang Liu, Bee Luan Khoo, Song Lin Chua</t>
         </is>
       </c>
-      <c r="I147" s="3" t="inlineStr">
+      <c r="J147" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsptsci.3c00354</t>
         </is>
@@ -7125,10 +7861,15 @@
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I148" s="3" t="inlineStr">
+        <is>
           <t>Chuan Li, Xiaohong Zhu, Donghong Wang, Shuo Yang, Rong Zhang, Pei Li, Jun Fan, Hongfei Li ...</t>
         </is>
       </c>
-      <c r="I148" s="3" t="inlineStr">
+      <c r="J148" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.3c08398</t>
         </is>
@@ -7170,10 +7911,15 @@
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="inlineStr">
+        <is>
           <t>Yuchen Xiong, Mohammed A H Alnoud, Hamid Ali, Ijaz Ali, Saleem Ahmad, Munir Ullah Khan, Syed Shams Ul Hassan, Muhammad Majid ...</t>
         </is>
       </c>
-      <c r="I149" s="3" t="inlineStr">
+      <c r="J149" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cpcardiol.2024.102390</t>
         </is>
@@ -7215,10 +7961,15 @@
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
           <t>Xiaorui Jiang, Mohammed A H Alnoud, Hamid Ali, Ijaz Ali, Talib Hussain, Munir Ullah Khan, Safir Ullah Khan, Muhammad Shehzad Khan ...</t>
         </is>
       </c>
-      <c r="I150" s="3" t="inlineStr">
+      <c r="J150" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cpcardiol.2024.102397</t>
         </is>
@@ -7260,10 +8011,15 @@
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr">
+        <is>
           <t>Se-Weon Park, Joseph H C Lai, Xiongqi Han, Vivian W M Leung, Peng Xiao, Jianpan Huang, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I151" s="3" t="inlineStr">
+      <c r="J151" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/pharmaceutics16010101</t>
         </is>
@@ -7305,10 +8061,15 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
           <t>Dengfeng Li, Jingkun Zhou, Zichen Zhao, Xingcan Huang, Hu Li, Qing'ao Qu, Changfei Zhou, Kuanming Yao ...</t>
         </is>
       </c>
-      <c r="I152" s="3" t="inlineStr">
+      <c r="J152" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adk6301</t>
         </is>
@@ -7350,10 +8111,15 @@
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="inlineStr">
+        <is>
           <t>Russell W Chan, Bradley Jay Edelman, Shui Ying Tsang, Kai Gao, Albert Cheung-Hoi Yu</t>
         </is>
       </c>
-      <c r="I153" s="3" t="inlineStr">
+      <c r="J153" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/978-3-031-69188-1_10</t>
         </is>
@@ -7395,10 +8161,15 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="inlineStr">
+        <is>
           <t>Zilin Chen, Joseph H C Lai, Jiadi Xu, Hao Zhang, Jianpan Huang, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I154" s="3" t="inlineStr">
+      <c r="J154" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.5093</t>
         </is>
@@ -7440,10 +8211,15 @@
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="inlineStr">
+        <is>
           <t>Chuanyin Xiong, Weihua Dang, Qi Yang, Qiusheng Zhou, Mengxia Shen, Qiancheng Xiong, Meng An, Xue Jiang ...</t>
         </is>
       </c>
-      <c r="I155" s="3" t="inlineStr">
+      <c r="J155" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202305962</t>
         </is>
@@ -7485,10 +8261,15 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="inlineStr">
+        <is>
           <t>Guangyao Zhao, Kuanming Yao, Yiming Liu, Xingcan Huang, Xinge Yu</t>
         </is>
       </c>
-      <c r="I156" s="3" t="inlineStr">
+      <c r="J156" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.7507/1001-5515.202210035</t>
         </is>
@@ -7530,10 +8311,15 @@
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
           <t>Yufei Zhang, Jingjing Fu, Yichun Ding, Aijaz Ahmed Babar, Xian Song, Fan Chen, Xinge Yu, Zijian Zheng</t>
         </is>
       </c>
-      <c r="I157" s="3" t="inlineStr">
+      <c r="J157" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202311633</t>
         </is>
@@ -7575,10 +8361,15 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
           <t>Muhammad Suleman, Shahid Ullah Khan, Talib Hussain, Munir Ullah Khan, Syed Shamsul Hassan, Muhammad Majid, Safir Ullah Khan, Muhammad Shehzad Khan ...</t>
         </is>
       </c>
-      <c r="I158" s="3" t="inlineStr">
+      <c r="J158" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cpcardiol.2023.102353</t>
         </is>
@@ -7620,10 +8411,15 @@
       </c>
       <c r="H159" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I159" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Yue Hou, Yiqiao Wang, Zhiquan Wei, Ao Chen, Pei Li, Zhaodong Huang, Nan Li ...</t>
         </is>
       </c>
-      <c r="I159" s="3" t="inlineStr">
+      <c r="J159" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202309330</t>
         </is>
@@ -7665,10 +8461,15 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I160" s="3" t="inlineStr">
+        <is>
           <t>Hu Hong, Jiaxiong Zhu, Yiqiao Wang, Zhiquan Wei, Xun Guo, Shuo Yang, Rong Zhang, Huilin Cui ...</t>
         </is>
       </c>
-      <c r="I160" s="3" t="inlineStr">
+      <c r="J160" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202308210</t>
         </is>
@@ -7710,10 +8511,15 @@
       </c>
       <c r="H161" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="inlineStr">
+        <is>
           <t>Xinliang Li, Shixun Wang, Dechao Zhang, Pei Li, Ze Chen, Ao Chen, Zhaodong Huang, Guojin Liang ...</t>
         </is>
       </c>
-      <c r="I161" s="3" t="inlineStr">
+      <c r="J161" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202304557</t>
         </is>
@@ -7755,10 +8561,15 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I162" s="3" t="inlineStr">
+        <is>
           <t>Qing Li, Hu Hong, Jiaxiong Zhu, Zhuoxi Wu, Chuan Li, Donghong Wang, Pei Li, Yuwei Zhao ...</t>
         </is>
       </c>
-      <c r="I162" s="3" t="inlineStr">
+      <c r="J162" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.3c07848</t>
         </is>
@@ -7800,10 +8611,15 @@
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I163" s="3" t="inlineStr">
+        <is>
           <t>Peter H Charlton, John Allen, Raquel Bailón, Stephanie Baker, Joachim A Behar, Fei Chen, Gari D Clifford, David A Clifton ...</t>
         </is>
       </c>
-      <c r="I163" s="3" t="inlineStr">
+      <c r="J163" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1088/1361-6579/acead2</t>
         </is>
@@ -7845,10 +8661,15 @@
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I164" s="3" t="inlineStr">
+        <is>
           <t>Ahsan Riaz Khan, Mohammed A H Alnoud, Hamid Ali, Ijaz Ali, Saleem Ahmad, Syed Shams Ul Hassan, Abdul Lateef Shaikh, Talib Hussain ...</t>
         </is>
       </c>
-      <c r="I164" s="3" t="inlineStr">
+      <c r="J164" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cpcardiol.2023.102222</t>
         </is>
@@ -7890,10 +8711,15 @@
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I165" s="3" t="inlineStr">
+        <is>
           <t>Hu Li, Huarui Gong, Tsz Hung Wong, Jingkun Zhou, Yuqiong Wang, Long Lin, Ying Dou, Huiling Jia ...</t>
         </is>
       </c>
-      <c r="I165" s="3" t="inlineStr">
+      <c r="J165" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-023-43189-z</t>
         </is>
@@ -7935,10 +8761,15 @@
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I166" s="3" t="inlineStr">
+        <is>
           <t>Muhammad Shehzad Khan, Shahid Ullah Khan, Safir Ullah Khan, Muhammad Suleman, Rafi U Shan Ahmad, Munir Ullah Khan, Jehad Zuhair Tayyeb, Sergio Crovella ...</t>
         </is>
       </c>
-      <c r="I166" s="3" t="inlineStr">
+      <c r="J166" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cpcardiol.2023.102189</t>
         </is>
@@ -7980,10 +8811,15 @@
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I167" s="3" t="inlineStr">
+        <is>
           <t>Wooyoung Park, Yiming Liu, Yanli Jiao, Rui Shi, Jin Nan, Chun Ki Yiu, Xingcan Huang, Yao Chen ...</t>
         </is>
       </c>
-      <c r="I167" s="3" t="inlineStr">
+      <c r="J167" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsnano.3c08287</t>
         </is>
@@ -8025,10 +8861,15 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="inlineStr">
+        <is>
           <t>Jianpan Huang, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I168" s="3" t="inlineStr">
+      <c r="J168" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/jmri.29096</t>
         </is>
@@ -8070,10 +8911,15 @@
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I169" s="3" t="inlineStr">
+        <is>
           <t>Rong Zhang, Hu Hong, Xinghui Liu, Shaoce Zhang, Chuan Li, Huilin Cui, Yanbo Wang, Jiahua Liu ...</t>
         </is>
       </c>
-      <c r="I169" s="3" t="inlineStr">
+      <c r="J169" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202309930</t>
         </is>
@@ -8115,10 +8961,15 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I170" s="3" t="inlineStr">
+        <is>
           <t>Yanbo Wang, Jiaxiong Zhu, Ao Chen, Xun Guo, Huilin Cui, Ze Chen, Yue Hou, Zhaodong Huang ...</t>
         </is>
       </c>
-      <c r="I170" s="3" t="inlineStr">
+      <c r="J170" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202303165</t>
         </is>
@@ -8160,10 +9011,15 @@
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="inlineStr">
+        <is>
           <t>Kexin Wang, Jianpan Huang, Licheng Ju, Su Xu, Rao P Gullapalli, Yajie Liang, Joshua Rogers, Yuguo Li ...</t>
         </is>
       </c>
-      <c r="I171" s="3" t="inlineStr">
+      <c r="J171" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/mrm.29876</t>
         </is>
@@ -8205,10 +9061,15 @@
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="inlineStr">
+        <is>
           <t>Yale Yang, Dengfeng Li, Yanhua Sun, Mengge Wu, Jingyou Su, Ying Li, Xinge Yu, Lu Li ...</t>
         </is>
       </c>
-      <c r="I172" s="3" t="inlineStr">
+      <c r="J172" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41378-023-00592-2</t>
         </is>
@@ -8250,10 +9111,15 @@
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="inlineStr">
+        <is>
           <t>Chenyang Wu, Xuezhi Qin, Huanxi Zheng, Zhenyu Xu, Yuxin Song, Yuankai Jin, Huanhuan Zhang, Jiaying Mo ...</t>
         </is>
       </c>
-      <c r="I173" s="3" t="inlineStr">
+      <c r="J173" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smll.202304635</t>
         </is>
@@ -8295,10 +9161,15 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
           <t>Haojun Hua, Shangjie Zou, Zhiqiang Ma, Wang Guo, Ching Yin Fong, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I174" s="3" t="inlineStr">
+      <c r="J174" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41378-023-00577-1</t>
         </is>
@@ -8340,10 +9211,15 @@
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="inlineStr">
+        <is>
           <t>Xinran Jiang, Han Wu, Ao Xiao, Ya Huang, Xinge Yu, Lingqian Chang</t>
         </is>
       </c>
-      <c r="I175" s="3" t="inlineStr">
+      <c r="J175" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smtd.202301068</t>
         </is>
@@ -8385,10 +9261,15 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="inlineStr">
+        <is>
           <t>Xinliang Li, Yanlei Wang, Junfeng Lu, Shimei Li, Pei Li, Zhaodong Huang, Guojin Liang, Hongyan He ...</t>
         </is>
       </c>
-      <c r="I176" s="3" t="inlineStr">
+      <c r="J176" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202310168</t>
         </is>
@@ -8430,10 +9311,15 @@
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Shengnan Wang, Zhiquan Wei, Yiqiao Wang, Zhuoxi Wu, Yue Hou, Jiaxiong Zhu, Yanbo Wang ...</t>
         </is>
       </c>
-      <c r="I177" s="3" t="inlineStr">
+      <c r="J177" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/jacs.3c06488</t>
         </is>
@@ -8475,10 +9361,15 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I178" s="3" t="inlineStr">
+        <is>
           <t>Chuan Li, Qing Li, Zhuoxi Wu, Yiqiao Wang, Rong Zhang, Huilin Cui, Yue Hou, Jiahua Liu ...</t>
         </is>
       </c>
-      <c r="I178" s="3" t="inlineStr">
+      <c r="J178" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202304878</t>
         </is>
@@ -8520,10 +9411,15 @@
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I179" s="3" t="inlineStr">
+        <is>
           <t>Lijing Kang, Juanjuan Yi, Chi-Wai Lau, Lei He, Qinghua Chen, Suowen Xu, Jun Li, Yin Xia ...</t>
         </is>
       </c>
-      <c r="I179" s="3" t="inlineStr">
+      <c r="J179" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/antiox12091681</t>
         </is>
@@ -8565,10 +9461,15 @@
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I180" s="3" t="inlineStr">
+        <is>
           <t>Zainab Riaz, Bangul Khan, Saad Abdullah, Samiullah Khan, Md Shohidul Islam</t>
         </is>
       </c>
-      <c r="I180" s="3" t="inlineStr">
+      <c r="J180" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/bioengineering10080981</t>
         </is>
@@ -8610,10 +9511,15 @@
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="inlineStr">
+        <is>
           <t>Jian Li, Huiling Jia, Jingkun Zhou, Xingcan Huang, Long Xu, Shengxin Jia, Zhan Gao, Kuanming Yao ...</t>
         </is>
       </c>
-      <c r="I181" s="3" t="inlineStr">
+      <c r="J181" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-023-40763-3</t>
         </is>
@@ -8655,10 +9561,15 @@
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
           <t>Ying Wang, Jimin Fu, Haibo Hu, Derek Ho</t>
         </is>
       </c>
-      <c r="I182" s="3" t="inlineStr">
+      <c r="J182" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsami.3c08512</t>
         </is>
@@ -8700,10 +9611,15 @@
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I183" s="3" t="inlineStr">
+        <is>
           <t>Yu Zhang, Yuefeng Zhang, Zhiyuan Zeng, Derek Ho</t>
         </is>
       </c>
-      <c r="I183" s="3" t="inlineStr">
+      <c r="J183" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/d3mh00339f</t>
         </is>
@@ -8745,10 +9661,15 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I184" s="3" t="inlineStr">
+        <is>
           <t>Shumaila Noreen, Ibrar Muhammad Khan, Muhammad Shehzad Khan, Bibi Zarnaab, Iram Gul, Muhammad Zahoor Khan, Waqar Azeem Jadoon, Shehzad Ghayyur ...</t>
         </is>
       </c>
-      <c r="I184" s="3" t="inlineStr">
+      <c r="J184" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s11356-023-28515-8</t>
         </is>
@@ -8790,10 +9711,15 @@
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="inlineStr">
+        <is>
           <t>Yatian Fu, Yanlin Deng, Jing Zhang, Song Lin Chua, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I185" s="3" t="inlineStr">
+      <c r="J185" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.actbio.2023.06.028</t>
         </is>
@@ -8835,10 +9761,15 @@
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
           <t>Kaiwen Wan, Lei Li, Dengqiang Jia, Shangqi Gao, Wei Qian, Yingzhi Wu, Huandong Lin, Xiongzheng Mu ...</t>
         </is>
       </c>
-      <c r="I186" s="3" t="inlineStr">
+      <c r="J186" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.media.2023.102875</t>
         </is>
@@ -8880,10 +9811,15 @@
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I187" s="3" t="inlineStr">
+        <is>
           <t>George S Stergiou, Alberto P Avolio, Paolo Palatini, Konstantinos G Kyriakoulis, Aletta E Schutte, Stephan Mieke, Anastasios Kollias, Gianfranco Parati ...</t>
         </is>
       </c>
-      <c r="I187" s="3" t="inlineStr">
+      <c r="J187" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1097/HJH.0000000000003483</t>
         </is>
@@ -8925,10 +9861,15 @@
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I188" s="3" t="inlineStr">
+        <is>
           <t>Zhaodong Huang, Xinliang Li, Ze Chen, Pei Li, Xiulei Ji, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I188" s="3" t="inlineStr">
+      <c r="J188" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41570-023-00506-w</t>
         </is>
@@ -8970,10 +9911,15 @@
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I189" s="3" t="inlineStr">
+        <is>
           <t>Yeping Ma, Yanlin Deng, Haojun Hua, Bee Luan Khoo, Song Lin Chua</t>
         </is>
       </c>
-      <c r="I189" s="3" t="inlineStr">
+      <c r="J189" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41396-023-01446-5</t>
         </is>
@@ -9015,10 +9961,15 @@
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I190" s="3" t="inlineStr">
+        <is>
           <t>Jianpan Huang, Joseph H C Lai, Xiongqi Han, Zilin Chen, Peng Xiao, Yang Liu, Lin Chen, Jiadi Xu ...</t>
         </is>
       </c>
-      <c r="I190" s="3" t="inlineStr">
+      <c r="J190" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.4962</t>
         </is>
@@ -9060,10 +10011,15 @@
       </c>
       <c r="H191" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I191" s="3" t="inlineStr">
+        <is>
           <t>Qiuna Zhuang, Kuanming Yao, Mengge Wu, Zhuogui Lei, Fan Chen, Jiyu Li, Quanjing Mei, Yingying Zhou ...</t>
         </is>
       </c>
-      <c r="I191" s="3" t="inlineStr">
+      <c r="J191" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adg8602</t>
         </is>
@@ -9105,10 +10061,15 @@
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I192" s="3" t="inlineStr">
+        <is>
           <t>Lei Zhao, Cunman Liang, Yan Huang, Guodong Zhou, Yiqun Xiao, Nan Ji, Yuan-Ting Zhang, Ni Zhao</t>
         </is>
       </c>
-      <c r="I192" s="3" t="inlineStr">
+      <c r="J192" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41746-023-00835-6</t>
         </is>
@@ -9150,10 +10111,15 @@
       </c>
       <c r="H193" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I193" s="3" t="inlineStr">
+        <is>
           <t>Xiao Yang, Simin Gao, Boguang Yang, Zhinan Yang, Feng Lou, Pei Huang, Pengchao Zhao, Jiaxin Guo ...</t>
         </is>
       </c>
-      <c r="I193" s="3" t="inlineStr">
+      <c r="J193" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202302272</t>
         </is>
@@ -9195,10 +10161,15 @@
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I194" s="3" t="inlineStr">
+        <is>
           <t>Jiahui He, Yuyue Zhang, Xinge Yu, Chenjie Xu</t>
         </is>
       </c>
-      <c r="I194" s="3" t="inlineStr">
+      <c r="J194" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.apsb.2023.05.009</t>
         </is>
@@ -9240,10 +10211,15 @@
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I195" s="3" t="inlineStr">
+        <is>
           <t>Yiming Liu, Chun Ki Yiu, Zhao Zhao, Wooyoung Park, Rui Shi, Xingcan Huang, Yuyang Zeng, Kuan Wang ...</t>
         </is>
       </c>
-      <c r="I195" s="3" t="inlineStr">
+      <c r="J195" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-023-37678-4</t>
         </is>
@@ -9285,10 +10261,15 @@
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I196" s="3" t="inlineStr">
+        <is>
           <t>Bangul Khan, Saad Abdullah, Samiullah Khan</t>
         </is>
       </c>
-      <c r="I196" s="3" t="inlineStr">
+      <c r="J196" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/mi14051005</t>
         </is>
@@ -9330,10 +10311,15 @@
       </c>
       <c r="H197" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I197" s="3" t="inlineStr">
+        <is>
           <t>Yu Wang, Bochun Liang, Jiaxiong Zhu, Geng Li, Qing Li, Ruquan Ye, Jun Fan, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I197" s="3" t="inlineStr">
+      <c r="J197" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202302583</t>
         </is>
@@ -9375,10 +10361,15 @@
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I198" s="3" t="inlineStr">
+        <is>
           <t>Pei Li, Yiqiao Wang, Qi Xiong, Yue Hou, Shuo Yang, Huilin Cui, Jiaxiong Zhu, Xinliang Li ...</t>
         </is>
       </c>
-      <c r="I198" s="3" t="inlineStr">
+      <c r="J198" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202303292</t>
         </is>
@@ -9420,10 +10411,15 @@
       </c>
       <c r="H199" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I199" s="3" t="inlineStr">
+        <is>
           <t>Qing Li, Hu Hong, Xun Guo, Jiaxiong Zhu, Yue Hou, Chao Liu, Donghong Wang, Guojin Liang ...</t>
         </is>
       </c>
-      <c r="I199" s="3" t="inlineStr">
+      <c r="J199" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.scib.2023.04.020</t>
         </is>
@@ -9465,10 +10461,15 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I200" s="3" t="inlineStr">
+        <is>
           <t>Lei Liu, Yuan-Ting Zhang, Wenyan Wang, Yifan Chen, Xiaorong Ding</t>
         </is>
       </c>
-      <c r="I200" s="3" t="inlineStr">
+      <c r="J200" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.compbiomed.2023.106900</t>
         </is>
@@ -9510,10 +10511,15 @@
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I201" s="3" t="inlineStr">
+        <is>
           <t>Jiyu Li, Yang Fu, Jingkun Zhou, Kuanming Yao, Xue Ma, Shouwei Gao, Zuankai Wang, Jian-Guo Dai ...</t>
         </is>
       </c>
-      <c r="I201" s="3" t="inlineStr">
+      <c r="J201" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.adg1837</t>
         </is>
@@ -9555,10 +10561,15 @@
       </c>
       <c r="H202" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I202" s="3" t="inlineStr">
+        <is>
           <t>Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I202" s="3" t="inlineStr">
+      <c r="J202" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.ebiom.2023.104554</t>
         </is>
@@ -9600,10 +10611,15 @@
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
           <t>Yu Wang, Tairan Wang, Shuyu Bu, Jiaxiong Zhu, Yanbo Wang, Rong Zhang, Hu Hong, Wenjun Zhang ...</t>
         </is>
       </c>
-      <c r="I203" s="3" t="inlineStr">
+      <c r="J203" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-023-37524-7</t>
         </is>
@@ -9645,10 +10661,15 @@
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I204" s="3" t="inlineStr">
+        <is>
           <t>Guojin Liang, Zijie Tang, Bing Han, Jiaxiong Zhu, Ao Chen, Qing Li, Ze Chen, Zhaodong Huang ...</t>
         </is>
       </c>
-      <c r="I204" s="3" t="inlineStr">
+      <c r="J204" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202210051</t>
         </is>
@@ -9690,10 +10711,15 @@
       </c>
       <c r="H205" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr">
+        <is>
           <t>Wenqi Ouyang, Xiayi Xu, Wanping Lu, Ni Zhao, Fei Han, Shih-Chi Chen</t>
         </is>
       </c>
-      <c r="I205" s="3" t="inlineStr">
+      <c r="J205" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-023-37163-y</t>
         </is>
@@ -9735,10 +10761,15 @@
       </c>
       <c r="H206" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I206" s="3" t="inlineStr">
+        <is>
           <t>Zilin Chen, Jianpan Huang, Joseph H C Lai, Kai-Hei Tse, Jiadi Xu, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I206" s="3" t="inlineStr">
+      <c r="J206" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.4937</t>
         </is>
@@ -9780,10 +10811,15 @@
       </c>
       <c r="H207" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I207" s="3" t="inlineStr">
+        <is>
           <t>Xingcan Huang, Yiming Liu, Wooyoung Park, Jiyu Li, Jie Ma, Chun Ki Yiu, Qiang Zhang, Jian Li ...</t>
         </is>
       </c>
-      <c r="I207" s="3" t="inlineStr">
+      <c r="J207" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adhm.202202846</t>
         </is>
@@ -9825,10 +10861,15 @@
       </c>
       <c r="H208" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I208" s="3" t="inlineStr">
+        <is>
           <t>Mengge Wu, Kuanming Yao, Ningge Huang, Hu Li, Jingkun Zhou, Rui Shi, Jiyu Li, Xingcan Huang ...</t>
         </is>
       </c>
-      <c r="I208" s="3" t="inlineStr">
+      <c r="J208" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202300504</t>
         </is>
@@ -9870,10 +10911,15 @@
       </c>
       <c r="H209" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I209" s="3" t="inlineStr">
+        <is>
           <t>Ying Wang, Jimin Fu, Jiangang Xu, Haibo Hu, Derek Ho</t>
         </is>
       </c>
-      <c r="I209" s="3" t="inlineStr">
+      <c r="J209" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsami.2c22609</t>
         </is>
@@ -9915,10 +10961,15 @@
       </c>
       <c r="H210" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
           <t>Shan Wang, Shepherd Yuen Chan, Yanlin Deng, Bee Luan Khoo, Song Lin Chua</t>
         </is>
       </c>
-      <c r="I210" s="3" t="inlineStr">
+      <c r="J210" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jare.2023.02.011</t>
         </is>
@@ -9960,10 +11011,15 @@
       </c>
       <c r="H211" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I211" s="3" t="inlineStr">
+        <is>
           <t>Junjie Shi, Ke Mao, Qixiang Zhang, Zunyu Liu, Fei Long, Li Wen, Yixin Hou, Xinliang Li ...</t>
         </is>
       </c>
-      <c r="I211" s="3" t="inlineStr">
+      <c r="J211" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s40820-023-01023-7</t>
         </is>
@@ -10005,10 +11061,15 @@
       </c>
       <c r="H212" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
           <t>Shangjie Zou, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I212" s="3" t="inlineStr">
+      <c r="J212" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3389/fimmu.2023.1053793</t>
         </is>
@@ -10050,10 +11111,15 @@
       </c>
       <c r="H213" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
           <t>Shuai-Chen Wang, Binbin Zhang, Lijing Kang, Cunman Liang, Dongdong Chen, Guoqiang Liu, Xuyun Guo</t>
         </is>
       </c>
-      <c r="I213" s="3" t="inlineStr">
+      <c r="J213" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/s23042021</t>
         </is>
@@ -10095,10 +11161,15 @@
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
+        <is>
           <t>Yanlin Deng, Yatian Fu, Song Lin Chua, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I214" s="3" t="inlineStr">
+      <c r="J214" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smll.202205904</t>
         </is>
@@ -10140,10 +11211,15 @@
       </c>
       <c r="H215" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr">
+        <is>
           <t>Jiyu Li, Xingcan Huang, Yawen Yang, Jingkun Zhou, Kuanming Yao, Jian Li, Yingying Zhou, Meixi Li ...</t>
         </is>
       </c>
-      <c r="I215" s="3" t="inlineStr">
+      <c r="J215" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/btm2.10445</t>
         </is>
@@ -10185,10 +11261,15 @@
       </c>
       <c r="H216" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr">
+        <is>
           <t>Li Zou, Kisum Chu, Xuan He, Ye Li, Liangbin Zhou, Xiayi Xu, Wei-Hsin Liao, Ling Qin</t>
         </is>
       </c>
-      <c r="I216" s="3" t="inlineStr">
+      <c r="J216" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/bioengineering10010095</t>
         </is>
@@ -10230,10 +11311,15 @@
       </c>
       <c r="H217" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
           <t>Lok Hin Law, Jianpan Huang, Peng Xiao, Yang Liu, Zilin Chen, Joseph H C Lai, Xiongqi Han, Gerald W Y Cheng ...</t>
         </is>
       </c>
-      <c r="I217" s="3" t="inlineStr">
+      <c r="J217" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jconrel.2023.01.011</t>
         </is>
@@ -10275,10 +11361,15 @@
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I218" s="3" t="inlineStr">
+        <is>
           <t>Chuan Li, Shuo Yang, Ying Guo, Haiming Lv, Pei Li, Xiaofang Bai, Xuejin Li, Chunyi Zhi ...</t>
         </is>
       </c>
-      <c r="I218" s="3" t="inlineStr">
+      <c r="J218" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/smtd.202201448</t>
         </is>
@@ -10320,10 +11411,15 @@
       </c>
       <c r="H219" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr">
+        <is>
           <t>Dengfeng Li, Jingkun Zhou, Kuanming Yao, Sitong Liu, Jiahui He, Jingyou Su, Qing'ao Qu, Yuyu Gao ...</t>
         </is>
       </c>
-      <c r="I219" s="3" t="inlineStr">
+      <c r="J219" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.ade2450</t>
         </is>
@@ -10365,10 +11461,15 @@
       </c>
       <c r="H220" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
           <t>Fei Han, Songyun Gu, Aleks Klimas, Ni Zhao, Yongxin Zhao, Shih-Chi Chen</t>
         </is>
       </c>
-      <c r="I220" s="3" t="inlineStr">
+      <c r="J220" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/science.abm8420</t>
         </is>
@@ -10410,10 +11511,15 @@
       </c>
       <c r="H221" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
           <t>Peilin Fang, Xianglin Ji, Xi Zhao, Richard Yan-Do, Youyang Wan, Ying Wang, Yuanting Zhang, Peng Shi</t>
         </is>
       </c>
-      <c r="I221" s="3" t="inlineStr">
+      <c r="J221" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202207282</t>
         </is>
@@ -10455,10 +11561,15 @@
       </c>
       <c r="H222" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I222" s="3" t="inlineStr">
+        <is>
           <t>Xu Jing, Jieyu Wu, Caijuan Dong, Juan Gao, Takahiro Seki, Changil Kim, Egon Urgard, Kayoko Hosaka ...</t>
         </is>
       </c>
-      <c r="I222" s="3" t="inlineStr">
+      <c r="J222" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s42255-022-00697-4</t>
         </is>
@@ -10500,10 +11611,15 @@
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
           <t>Marko Gosak, Richard Yan-Do, Haopeng Lin, Patrick E MacDonald, Andraž Stožer</t>
         </is>
       </c>
-      <c r="I223" s="3" t="inlineStr">
+      <c r="J223" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.2337/db22-0004</t>
         </is>
@@ -10545,10 +11661,15 @@
       </c>
       <c r="H224" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I224" s="3" t="inlineStr">
+        <is>
           <t>Peng Xiao, Jianpan Huang, Xiongqi Han, Jacinth W S Cheu, Yang Liu, Lok Hin Law, Joseph H C Lai, Jiyu Li ...</t>
         </is>
       </c>
-      <c r="I224" s="3" t="inlineStr">
+      <c r="J224" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsami.2c10493</t>
         </is>
@@ -10590,10 +11711,15 @@
       </c>
       <c r="H225" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
           <t>Irfan Ahmed, Muhammad Shehzad Khan, Victor Ma, Hina Magsi, Renardi Gunawan, Abdul-Mojeed Olabisi Ilyas, Najeeb Ur Rehman Lashari, Naveed Wassan ...</t>
         </is>
       </c>
-      <c r="I225" s="3" t="inlineStr">
+      <c r="J225" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/bdi.13275</t>
         </is>
@@ -10635,10 +11761,15 @@
       </c>
       <c r="H226" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I226" s="3" t="inlineStr">
+        <is>
           <t>Joseph H C Lai, Jiaxin Liu, Tian Yang, Jianpan Huang, Yang Liu, Zilin Chen, Youngjin Lee, Gilberto K K Leung ...</t>
         </is>
       </c>
-      <c r="I226" s="3" t="inlineStr">
+      <c r="J226" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1161/STROKEAHA.122.040830</t>
         </is>
@@ -10680,10 +11811,15 @@
       </c>
       <c r="H227" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I227" s="3" t="inlineStr">
+        <is>
           <t>Yihai Cao</t>
         </is>
       </c>
-      <c r="I227" s="3" t="inlineStr">
+      <c r="J227" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1097/CM9.0000000000002406</t>
         </is>
@@ -10725,10 +11861,15 @@
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I228" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Tairan Wang, Yue Hou, Yanbo Wang, Zhaodong Huang, Huilin Cui, Jun Fan, Zengxia Pei ...</t>
         </is>
       </c>
-      <c r="I228" s="3" t="inlineStr">
+      <c r="J228" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202207682</t>
         </is>
@@ -10770,10 +11911,15 @@
       </c>
       <c r="H229" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I229" s="3" t="inlineStr">
+        <is>
           <t>Qingyun Huang, Cong Wu, Senlin Hou, Kuanming Yao, Hui Sun, Yufan Wang, Yikai Chen, Junhui Law ...</t>
         </is>
       </c>
-      <c r="I229" s="3" t="inlineStr">
+      <c r="J229" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adhm.202201404</t>
         </is>
@@ -10815,10 +11961,15 @@
       </c>
       <c r="H230" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I230" s="3" t="inlineStr">
+        <is>
           <t>Xi Zhao, Zixun Wang, Xianglin Ji, Shuyu Bu, Peilin Fang, Yuan Wang, Mingxue Wang, Yang Yang ...</t>
         </is>
       </c>
-      <c r="I230" s="3" t="inlineStr">
+      <c r="J230" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.biomaterials.2022.121869</t>
         </is>
@@ -10860,10 +12011,15 @@
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I231" s="3" t="inlineStr">
+        <is>
           <t>Fei Xu, Lingli Lin, Zihan Li, Qingqi Hong, Kunhong Liu, Qingqiang Wu, Qingde Li, Yinhuan Zheng ...</t>
         </is>
       </c>
-      <c r="I231" s="3" t="inlineStr">
+      <c r="J231" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.ymeth.2022.10.005</t>
         </is>
@@ -10905,10 +12061,15 @@
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I232" s="3" t="inlineStr">
+        <is>
           <t>Xinrong Li, Shih-Chi Chen, Jacque Pak Kan Ip</t>
         </is>
       </c>
-      <c r="I232" s="3" t="inlineStr">
+      <c r="J232" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/biom12101505</t>
         </is>
@@ -10950,10 +12111,15 @@
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I233" s="3" t="inlineStr">
+        <is>
           <t>Weibin Jia, Liling Liu, Min Li, Yuanmeng Zhou, Hang Zhou, Hongjuan Weng, Guofeng Gu, Min Xiao ...</t>
         </is>
       </c>
-      <c r="I233" s="3" t="inlineStr">
+      <c r="J233" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.actbio.2022.09.041</t>
         </is>
@@ -10995,10 +12161,15 @@
       </c>
       <c r="H234" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I234" s="3" t="inlineStr">
+        <is>
           <t>Hangjie Mo, Xiaojian Li, Bo Ouyang, Ge Fang, Yuanjun Jia</t>
         </is>
       </c>
-      <c r="I234" s="3" t="inlineStr">
+      <c r="J234" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.34133/2022/9759504</t>
         </is>
@@ -11040,10 +12211,15 @@
       </c>
       <c r="H235" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I235" s="3" t="inlineStr">
+        <is>
           <t>Jiao Suo, Yifan Liu, Cong Wu, Meng Chen, Qingyun Huang, Yiming Liu, Kuanming Yao, Yangbin Chen ...</t>
         </is>
       </c>
-      <c r="I235" s="3" t="inlineStr">
+      <c r="J235" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202203565</t>
         </is>
@@ -11085,10 +12261,15 @@
       </c>
       <c r="H236" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I236" s="3" t="inlineStr">
+        <is>
           <t>Linda Knutsson, Xiang Xu, Peter C M van Zijl, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I236" s="3" t="inlineStr">
+      <c r="J236" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.4784</t>
         </is>
@@ -11130,10 +12311,15 @@
       </c>
       <c r="H237" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I237" s="3" t="inlineStr">
+        <is>
           <t>Yatian Fu, Shangjie Zou, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I237" s="3" t="inlineStr">
+      <c r="J237" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.xpro.2022.101584</t>
         </is>
@@ -11175,10 +12361,15 @@
       </c>
       <c r="H238" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I238" s="3" t="inlineStr">
+        <is>
           <t>Ya Huang, Hu Li, Tianli Hu, Jian Li, Chun Ki Yiu, Jingkun Zhou, Jiyu Li, Xingcan Huang ...</t>
         </is>
       </c>
-      <c r="I238" s="3" t="inlineStr">
+      <c r="J238" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.nanolett.2c01997</t>
         </is>
@@ -11220,10 +12411,15 @@
       </c>
       <c r="H239" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I239" s="3" t="inlineStr">
+        <is>
           <t>Yue Chen, Qiong Zhan, Jian Zhang, Wei Wang, Bee Luan Khoo, Zhen Liu, Siqi Wei, Junxin Niu ...</t>
         </is>
       </c>
-      <c r="I239" s="3" t="inlineStr">
+      <c r="J239" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.aca.2022.340151</t>
         </is>
@@ -11265,10 +12461,15 @@
       </c>
       <c r="H240" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I240" s="3" t="inlineStr">
+        <is>
           <t>Qing Li, Ao Chen, Donghong Wang, Yuwei Zhao, Xiaoqi Wang, Xu Jin, Bo Xiong, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I240" s="3" t="inlineStr">
+      <c r="J240" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41467-022-31461-7</t>
         </is>
@@ -11310,10 +12511,15 @@
       </c>
       <c r="H241" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I241" s="3" t="inlineStr">
+        <is>
           <t>Donghong Wang, Xun Guo, Ze Chen, Yuwei Zhao, Qing Li, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I241" s="3" t="inlineStr">
+      <c r="J241" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsami.2c06793</t>
         </is>
@@ -11355,10 +12561,15 @@
       </c>
       <c r="H242" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I242" s="3" t="inlineStr">
+        <is>
           <t>Huilin Cui, Tairan Wang, Zhaodong Huang, Guojin Liang, Ze Chen, Ao Chen, Donghong Wang, Qi Yang ...</t>
         </is>
       </c>
-      <c r="I242" s="3" t="inlineStr">
+      <c r="J242" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202203453</t>
         </is>
@@ -11400,10 +12611,15 @@
       </c>
       <c r="H243" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I243" s="3" t="inlineStr">
+        <is>
           <t>Xudong Lin, Tianying Sun, Minghui Tang, Anqi Yang, Richard Yan-Do, Da Chen, Yaobin Gao, Xin Duan ...</t>
         </is>
       </c>
-      <c r="I243" s="3" t="inlineStr">
+      <c r="J243" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adhm.202200304</t>
         </is>
@@ -11445,10 +12661,15 @@
       </c>
       <c r="H244" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I244" s="3" t="inlineStr">
+        <is>
           <t>Qing Li, Donghong Wang, Boxun Yan, Yuwei Zhao, Jun Fan, Chunyi Zhi</t>
         </is>
       </c>
-      <c r="I244" s="3" t="inlineStr">
+      <c r="J244" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202202780</t>
         </is>
@@ -11490,10 +12711,15 @@
       </c>
       <c r="H245" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I245" s="3" t="inlineStr">
+        <is>
           <t>Xingcan Huang, Hu Li, Jiyu Li, Libei Huang, Kuanming Yao, Chun Ki Yiu, Yiming Liu, Tsz Hung Wong ...</t>
         </is>
       </c>
-      <c r="I245" s="3" t="inlineStr">
+      <c r="J245" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.nanolett.2c00864</t>
         </is>
@@ -11535,10 +12761,15 @@
       </c>
       <c r="H246" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I246" s="3" t="inlineStr">
+        <is>
           <t>Xi Zhao, Xianglin Ji, Jin Qu, Kai Xie, Zixun Wang, Peilin Fang, Yuan Wang, Youyang Wan ...</t>
         </is>
       </c>
-      <c r="I246" s="3" t="inlineStr">
+      <c r="J246" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/jacs.2c01036</t>
         </is>
@@ -11580,10 +12811,15 @@
       </c>
       <c r="H247" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I247" s="3" t="inlineStr">
+        <is>
           <t>Yang Sylvia Liu, Yanlin Deng, Chun Kwan Chen, Bee Luan Khoo, Song Lin Chua</t>
         </is>
       </c>
-      <c r="I247" s="3" t="inlineStr">
+      <c r="J247" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jhazmat.2022.128572</t>
         </is>
@@ -11625,10 +12861,15 @@
       </c>
       <c r="H248" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I248" s="3" t="inlineStr">
+        <is>
           <t>Jianpan Huang, Zilin Chen, Se-Weon Park, Joseph H C Lai, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I248" s="3" t="inlineStr">
+      <c r="J248" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/pharmaceutics14020451</t>
         </is>
@@ -11670,10 +12911,15 @@
       </c>
       <c r="H249" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I249" s="3" t="inlineStr">
+        <is>
           <t>Wei Li, Yunlan Zhou, Yanlin Deng, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I249" s="3" t="inlineStr">
+      <c r="J249" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/cancers14030818</t>
         </is>
@@ -11715,10 +12961,15 @@
       </c>
       <c r="H250" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I250" s="3" t="inlineStr">
+        <is>
           <t>Yiming Liu, Xingcan Huang, Jingkun Zhou, Chun Ki Yiu, Zhen Song, Wei Huang, Sina Khazaee Nejad, Hu Li ...</t>
         </is>
       </c>
-      <c r="I250" s="3" t="inlineStr">
+      <c r="J250" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202104635</t>
         </is>
@@ -11760,10 +13011,15 @@
       </c>
       <c r="H251" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I251" s="3" t="inlineStr">
+        <is>
           <t>Yiming Liu, Chunki Yiu, Zhen Song, Ya Huang, Kuanming Yao, Tszhung Wong, Jingkun Zhou, Ling Zhao ...</t>
         </is>
       </c>
-      <c r="I251" s="3" t="inlineStr">
+      <c r="J251" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1126/sciadv.abl6700</t>
         </is>
@@ -11805,10 +13061,15 @@
       </c>
       <c r="H252" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I252" s="3" t="inlineStr">
+        <is>
           <t>Xinliang Li, Yanlei Wang, Ze Chen, Pei Li, Guojin Liang, Zhaodong Huang, Qi Yang, Ao Chen ...</t>
         </is>
       </c>
-      <c r="I252" s="3" t="inlineStr">
+      <c r="J252" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202113576</t>
         </is>
@@ -11850,10 +13111,15 @@
       </c>
       <c r="H253" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I253" s="3" t="inlineStr">
+        <is>
           <t>Shangjie Zou, Bee Luan Khoo</t>
         </is>
       </c>
-      <c r="I253" s="3" t="inlineStr">
+      <c r="J253" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.gendis.2021.12.001</t>
         </is>
@@ -11895,10 +13161,15 @@
       </c>
       <c r="H254" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I254" s="3" t="inlineStr">
+        <is>
           <t>Qi Yang, Liang Li, Tanveer Hussain, Donghong Wang, Lan Hui, Ying Guo, Guojin Liang, Xinliang Li ...</t>
         </is>
       </c>
-      <c r="I254" s="3" t="inlineStr">
+      <c r="J254" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/anie.202112304</t>
         </is>
@@ -11940,10 +13211,15 @@
       </c>
       <c r="H255" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I255" s="3" t="inlineStr">
+        <is>
           <t>Junyang Li, Lei Fan, Yanfang Li, Tanyong Wei, Cheng Wang, Feng Li, Hua Tian, Dong Sun</t>
         </is>
       </c>
-      <c r="I255" s="3" t="inlineStr">
+      <c r="J255" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/mi12121572</t>
         </is>
@@ -11985,10 +13261,15 @@
       </c>
       <c r="H256" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I256" s="3" t="inlineStr">
+        <is>
           <t>Zhaodong Huang, Tairan Wang, Xinliang Li, Huilin Cui, Guojin Liang, Qi Yang, Ze Chen, Ao Chen ...</t>
         </is>
       </c>
-      <c r="I256" s="3" t="inlineStr">
+      <c r="J256" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202106180</t>
         </is>
@@ -12030,10 +13311,15 @@
       </c>
       <c r="H257" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I257" s="3" t="inlineStr">
+        <is>
           <t>Jianpan Huang, Joseph H C Lai, Xiongqi Han, Zilin Chen, Peng Xiao, Yang Liu, Lin Chen, Jiadi Xu ...</t>
         </is>
       </c>
-      <c r="I257" s="3" t="inlineStr">
+      <c r="J257" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/nbm.4640</t>
         </is>
@@ -12075,10 +13361,15 @@
       </c>
       <c r="H258" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I258" s="3" t="inlineStr">
+        <is>
           <t>Wooyoung Park, Chunki Yiu, Yiming Liu, Tsz Hung Wong, Xingcan Huang, Jingkun Zhou, Jian Li, Kuanming Yao ...</t>
         </is>
       </c>
-      <c r="I258" s="3" t="inlineStr">
+      <c r="J258" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/bios11110435</t>
         </is>
@@ -12120,10 +13411,15 @@
       </c>
       <c r="H259" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I259" s="3" t="inlineStr">
+        <is>
           <t>Jianpan Huang, Jiadi Xu, Joseph H C Lai, Zilin Chen, Chi Yan Lee, Henry K F Mak, Koon Ho Chan, Kannie W Y Chan</t>
         </is>
       </c>
-      <c r="I259" s="3" t="inlineStr">
+      <c r="J259" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.nicl.2021.102867</t>
         </is>
@@ -12165,10 +13461,15 @@
       </c>
       <c r="H260" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I260" s="3" t="inlineStr">
+        <is>
           <t>Dengfeng Li, Jiahui He, Zhen Song, Kuanming Yao, Mengge Wu, Haoran Fu, Yiming Liu, Zhan Gao ...</t>
         </is>
       </c>
-      <c r="I260" s="3" t="inlineStr">
+      <c r="J260" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41378-021-00301-x</t>
         </is>
@@ -12210,10 +13511,15 @@
       </c>
       <c r="H261" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I261" s="3" t="inlineStr">
+        <is>
           <t>Jianpan Huang, Joseph H C Lai, Kai-Hei Tse, Gerald W Y Cheng, Yang Liu, Zilin Chen, Xiongqi Han, Lin Chen ...</t>
         </is>
       </c>
-      <c r="I261" s="3" t="inlineStr">
+      <c r="J261" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/mrm.29044</t>
         </is>
@@ -12255,10 +13561,15 @@
       </c>
       <c r="H262" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I262" s="3" t="inlineStr">
+        <is>
           <t>Ze Chen, Chuan Li, Qi Yang, Donghong Wang, Xinliang Li, Zhaodong Huang, Guojin Liang, Ao Chen ...</t>
         </is>
       </c>
-      <c r="I262" s="3" t="inlineStr">
+      <c r="J262" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202105426</t>
         </is>
@@ -12300,10 +13611,15 @@
       </c>
       <c r="H263" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I263" s="3" t="inlineStr">
+        <is>
           <t>Wenhao Yan, Longtao Ma, Jiangang Xu, Ying Guo, Haibo Hu, Chunyi Zhi, Derek Ho</t>
         </is>
       </c>
-      <c r="I263" s="3" t="inlineStr">
+      <c r="J263" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acsami.1c09255</t>
         </is>
@@ -12345,10 +13661,15 @@
       </c>
       <c r="H264" s="3" t="inlineStr">
         <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I264" s="3" t="inlineStr">
+        <is>
           <t>Yun Chen, Bin Xie, Junyu Long, Yicheng Kuang, Xin Chen, Maoxiang Hou, Jian Gao, Shuang Zhou ...</t>
         </is>
       </c>
-      <c r="I264" s="3" t="inlineStr">
+      <c r="J264" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/adma.202104290</t>
         </is>
@@ -12362,14 +13683,27 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Yellow highlight = past 30 days (4 papers)</t>
+          <t>Yellow = past 30 days (4 papers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Green = InnoHK acknowledgement only (no COCHE affiliation, 0 papers)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I266"/>
-  <mergeCells count="1">
-    <mergeCell ref="B266:I266"/>
+  <autoFilter ref="A1:J267"/>
+  <mergeCells count="2">
+    <mergeCell ref="B267:J267"/>
+    <mergeCell ref="B266:J266"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
All-English README with explicit ⭐ Dual-Channel explanation
- README now explains ⭐ = BOTH COCHE affiliation + InnoHK/ITC acknowledgement
- All titles and labels in English (no Chinese)
- Excel legend and status labels also in English
- Clarity for ITC KPI reporting compliance
</commit_message>
<xml_diff>
--- a/COCHE_Papers.xlsx
+++ b/COCHE_Papers.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
@@ -4468,7 +4468,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4868,7 +4868,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
@@ -4968,7 +4968,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -5068,7 +5068,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -5118,7 +5118,7 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
@@ -5468,7 +5468,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I101" s="3" t="inlineStr">
@@ -5568,7 +5568,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>⭐ 双满足</t>
+          <t>⭐ Dual-Channel</t>
         </is>
       </c>
       <c r="I104" s="3" t="inlineStr">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I106" s="3" t="inlineStr">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5864,7 +5864,7 @@
       <c r="G108" s="4" t="inlineStr"/>
       <c r="H108" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I108" s="4" t="inlineStr">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="H110" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I110" s="4" t="inlineStr">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I111" s="4" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="H112" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I112" s="4" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="H114" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I114" s="4" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I115" s="4" t="inlineStr">
@@ -6260,7 +6260,7 @@
       <c r="G116" s="4" t="inlineStr"/>
       <c r="H116" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I116" s="4" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="H117" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I117" s="4" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="H118" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I118" s="4" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="H119" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I119" s="4" t="inlineStr">
@@ -6456,7 +6456,7 @@
       <c r="G120" s="4" t="inlineStr"/>
       <c r="H120" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I120" s="4" t="inlineStr">
@@ -6506,7 +6506,7 @@
       </c>
       <c r="H121" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I121" s="4" t="inlineStr">
@@ -6552,7 +6552,7 @@
       <c r="G122" s="4" t="inlineStr"/>
       <c r="H122" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I122" s="4" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="H123" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I123" s="4" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="H124" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I124" s="4" t="inlineStr">
@@ -6702,7 +6702,7 @@
       </c>
       <c r="H125" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I125" s="4" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="H126" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I126" s="4" t="inlineStr">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="H127" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I127" s="4" t="inlineStr">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="H128" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I128" s="4" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="H129" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I129" s="4" t="inlineStr">
@@ -6952,7 +6952,7 @@
       </c>
       <c r="H130" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I130" s="4" t="inlineStr">
@@ -6998,7 +6998,7 @@
       <c r="G131" s="4" t="inlineStr"/>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I131" s="4" t="inlineStr">
@@ -7048,7 +7048,7 @@
       </c>
       <c r="H132" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I132" s="4" t="inlineStr">
@@ -7094,7 +7094,7 @@
       <c r="G133" s="4" t="inlineStr"/>
       <c r="H133" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I133" s="4" t="inlineStr">
@@ -7144,7 +7144,7 @@
       </c>
       <c r="H134" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I134" s="4" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="H135" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I135" s="4" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="H136" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I136" s="4" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="H137" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I137" s="4" t="inlineStr">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="H138" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I138" s="4" t="inlineStr">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="H139" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I139" s="4" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="H140" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I140" s="4" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H141" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I141" s="4" t="inlineStr">
@@ -7544,7 +7544,7 @@
       </c>
       <c r="H142" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I142" s="4" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="H143" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I143" s="4" t="inlineStr">
@@ -7644,7 +7644,7 @@
       </c>
       <c r="H144" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I144" s="4" t="inlineStr">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="H145" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I145" s="4" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="H146" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I146" s="4" t="inlineStr">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="H147" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I147" s="4" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="H148" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I148" s="4" t="inlineStr">
@@ -7890,7 +7890,7 @@
       <c r="G149" s="4" t="inlineStr"/>
       <c r="H149" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I149" s="4" t="inlineStr">
@@ -7936,7 +7936,7 @@
       <c r="G150" s="4" t="inlineStr"/>
       <c r="H150" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I150" s="4" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="H151" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I151" s="4" t="inlineStr">
@@ -8036,7 +8036,7 @@
       </c>
       <c r="H152" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I152" s="4" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="H153" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I153" s="4" t="inlineStr">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="H154" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I154" s="4" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="H155" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I155" s="4" t="inlineStr">
@@ -8236,7 +8236,7 @@
       </c>
       <c r="H156" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I156" s="4" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="H157" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I157" s="4" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="H158" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I158" s="4" t="inlineStr">
@@ -8386,7 +8386,7 @@
       </c>
       <c r="H159" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I159" s="4" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="H160" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I160" s="4" t="inlineStr">
@@ -8482,7 +8482,7 @@
       <c r="G161" s="4" t="inlineStr"/>
       <c r="H161" s="4" t="inlineStr">
         <is>
-          <t>🏷 InnoHK</t>
+          <t>🏷 InnoHK-only</t>
         </is>
       </c>
       <c r="I161" s="4" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="H162" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I162" s="4" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H163" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I163" s="4" t="inlineStr">
@@ -8632,7 +8632,7 @@
       </c>
       <c r="H164" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I164" s="4" t="inlineStr">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="H165" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I165" s="4" t="inlineStr">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="H166" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I166" s="4" t="inlineStr">
@@ -8782,7 +8782,7 @@
       </c>
       <c r="H167" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I167" s="4" t="inlineStr">
@@ -8832,7 +8832,7 @@
       </c>
       <c r="H168" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I168" s="4" t="inlineStr">
@@ -8882,7 +8882,7 @@
       </c>
       <c r="H169" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I169" s="4" t="inlineStr">
@@ -8932,7 +8932,7 @@
       </c>
       <c r="H170" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I170" s="4" t="inlineStr">
@@ -8982,7 +8982,7 @@
       </c>
       <c r="H171" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I171" s="4" t="inlineStr">
@@ -9032,7 +9032,7 @@
       </c>
       <c r="H172" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I172" s="4" t="inlineStr">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="H173" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I173" s="4" t="inlineStr">
@@ -9132,7 +9132,7 @@
       </c>
       <c r="H174" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I174" s="4" t="inlineStr">
@@ -9182,7 +9182,7 @@
       </c>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I175" s="4" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="H176" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I176" s="4" t="inlineStr">
@@ -9282,7 +9282,7 @@
       </c>
       <c r="H177" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I177" s="4" t="inlineStr">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="H178" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I178" s="4" t="inlineStr">
@@ -9382,7 +9382,7 @@
       </c>
       <c r="H179" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I179" s="4" t="inlineStr">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="H180" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I180" s="4" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="H181" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I181" s="4" t="inlineStr">
@@ -9532,7 +9532,7 @@
       </c>
       <c r="H182" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I182" s="4" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="H183" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I183" s="4" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="H184" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I184" s="4" t="inlineStr">
@@ -9682,7 +9682,7 @@
       </c>
       <c r="H185" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I185" s="4" t="inlineStr">
@@ -9732,7 +9732,7 @@
       </c>
       <c r="H186" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I186" s="4" t="inlineStr">
@@ -9782,7 +9782,7 @@
       </c>
       <c r="H187" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I187" s="4" t="inlineStr">
@@ -9832,7 +9832,7 @@
       </c>
       <c r="H188" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I188" s="4" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H189" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I189" s="4" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="H190" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I190" s="4" t="inlineStr">
@@ -9982,7 +9982,7 @@
       </c>
       <c r="H191" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I191" s="4" t="inlineStr">
@@ -10032,7 +10032,7 @@
       </c>
       <c r="H192" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I192" s="4" t="inlineStr">
@@ -10082,7 +10082,7 @@
       </c>
       <c r="H193" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I193" s="4" t="inlineStr">
@@ -10132,7 +10132,7 @@
       </c>
       <c r="H194" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I194" s="4" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H195" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I195" s="4" t="inlineStr">
@@ -10232,7 +10232,7 @@
       </c>
       <c r="H196" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I196" s="4" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="H197" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I197" s="4" t="inlineStr">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="H198" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I198" s="4" t="inlineStr">
@@ -10382,7 +10382,7 @@
       </c>
       <c r="H199" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I199" s="4" t="inlineStr">
@@ -10432,7 +10432,7 @@
       </c>
       <c r="H200" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I200" s="4" t="inlineStr">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="H201" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I201" s="4" t="inlineStr">
@@ -10532,7 +10532,7 @@
       </c>
       <c r="H202" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I202" s="4" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="H203" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I203" s="4" t="inlineStr">
@@ -10632,7 +10632,7 @@
       </c>
       <c r="H204" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I204" s="4" t="inlineStr">
@@ -10682,7 +10682,7 @@
       </c>
       <c r="H205" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I205" s="4" t="inlineStr">
@@ -10732,7 +10732,7 @@
       </c>
       <c r="H206" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I206" s="4" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="H207" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I207" s="4" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="H208" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I208" s="4" t="inlineStr">
@@ -10882,7 +10882,7 @@
       </c>
       <c r="H209" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I209" s="4" t="inlineStr">
@@ -10932,7 +10932,7 @@
       </c>
       <c r="H210" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I210" s="4" t="inlineStr">
@@ -10982,7 +10982,7 @@
       </c>
       <c r="H211" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I211" s="4" t="inlineStr">
@@ -11032,7 +11032,7 @@
       </c>
       <c r="H212" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I212" s="4" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="H213" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I213" s="4" t="inlineStr">
@@ -11132,7 +11132,7 @@
       </c>
       <c r="H214" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I214" s="4" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="H215" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I215" s="4" t="inlineStr">
@@ -11232,7 +11232,7 @@
       </c>
       <c r="H216" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I216" s="4" t="inlineStr">
@@ -11282,7 +11282,7 @@
       </c>
       <c r="H217" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I217" s="4" t="inlineStr">
@@ -11332,7 +11332,7 @@
       </c>
       <c r="H218" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I218" s="4" t="inlineStr">
@@ -11382,7 +11382,7 @@
       </c>
       <c r="H219" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I219" s="4" t="inlineStr">
@@ -11432,7 +11432,7 @@
       </c>
       <c r="H220" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I220" s="4" t="inlineStr">
@@ -11482,7 +11482,7 @@
       </c>
       <c r="H221" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I221" s="4" t="inlineStr">
@@ -11532,7 +11532,7 @@
       </c>
       <c r="H222" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I222" s="4" t="inlineStr">
@@ -11582,7 +11582,7 @@
       </c>
       <c r="H223" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I223" s="4" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="H224" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I224" s="4" t="inlineStr">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="H225" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I225" s="4" t="inlineStr">
@@ -11732,7 +11732,7 @@
       </c>
       <c r="H226" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I226" s="4" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H227" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I227" s="4" t="inlineStr">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="H228" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I228" s="4" t="inlineStr">
@@ -11882,7 +11882,7 @@
       </c>
       <c r="H229" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I229" s="4" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="H230" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I230" s="4" t="inlineStr">
@@ -11982,7 +11982,7 @@
       </c>
       <c r="H231" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I231" s="4" t="inlineStr">
@@ -12032,7 +12032,7 @@
       </c>
       <c r="H232" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I232" s="4" t="inlineStr">
@@ -12082,7 +12082,7 @@
       </c>
       <c r="H233" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I233" s="4" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="H234" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I234" s="4" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="H235" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I235" s="4" t="inlineStr">
@@ -12232,7 +12232,7 @@
       </c>
       <c r="H236" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I236" s="4" t="inlineStr">
@@ -12282,7 +12282,7 @@
       </c>
       <c r="H237" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I237" s="4" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="H238" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I238" s="4" t="inlineStr">
@@ -12382,7 +12382,7 @@
       </c>
       <c r="H239" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I239" s="4" t="inlineStr">
@@ -12432,7 +12432,7 @@
       </c>
       <c r="H240" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I240" s="4" t="inlineStr">
@@ -12482,7 +12482,7 @@
       </c>
       <c r="H241" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I241" s="4" t="inlineStr">
@@ -12532,7 +12532,7 @@
       </c>
       <c r="H242" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I242" s="4" t="inlineStr">
@@ -12582,7 +12582,7 @@
       </c>
       <c r="H243" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I243" s="4" t="inlineStr">
@@ -12632,7 +12632,7 @@
       </c>
       <c r="H244" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I244" s="4" t="inlineStr">
@@ -12682,7 +12682,7 @@
       </c>
       <c r="H245" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I245" s="4" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="H246" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I246" s="4" t="inlineStr">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="H247" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I247" s="4" t="inlineStr">
@@ -12832,7 +12832,7 @@
       </c>
       <c r="H248" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I248" s="4" t="inlineStr">
@@ -12882,7 +12882,7 @@
       </c>
       <c r="H249" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I249" s="4" t="inlineStr">
@@ -12932,7 +12932,7 @@
       </c>
       <c r="H250" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I250" s="4" t="inlineStr">
@@ -12982,7 +12982,7 @@
       </c>
       <c r="H251" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I251" s="4" t="inlineStr">
@@ -13032,7 +13032,7 @@
       </c>
       <c r="H252" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I252" s="4" t="inlineStr">
@@ -13082,7 +13082,7 @@
       </c>
       <c r="H253" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I253" s="4" t="inlineStr">
@@ -13132,7 +13132,7 @@
       </c>
       <c r="H254" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I254" s="4" t="inlineStr">
@@ -13182,7 +13182,7 @@
       </c>
       <c r="H255" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I255" s="4" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="H256" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I256" s="4" t="inlineStr">
@@ -13282,7 +13282,7 @@
       </c>
       <c r="H257" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I257" s="4" t="inlineStr">
@@ -13332,7 +13332,7 @@
       </c>
       <c r="H258" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I258" s="4" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H259" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I259" s="4" t="inlineStr">
@@ -13432,7 +13432,7 @@
       </c>
       <c r="H260" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I260" s="4" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="H261" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I261" s="4" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="H262" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I262" s="4" t="inlineStr">
@@ -13582,7 +13582,7 @@
       </c>
       <c r="H263" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I263" s="4" t="inlineStr">
@@ -13632,7 +13632,7 @@
       </c>
       <c r="H264" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I264" s="4" t="inlineStr">
@@ -13682,7 +13682,7 @@
       </c>
       <c r="H265" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I265" s="4" t="inlineStr">
@@ -13732,7 +13732,7 @@
       </c>
       <c r="H266" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I266" s="4" t="inlineStr">
@@ -13782,7 +13782,7 @@
       </c>
       <c r="H267" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I267" s="4" t="inlineStr">
@@ -13832,7 +13832,7 @@
       </c>
       <c r="H268" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I268" s="4" t="inlineStr">
@@ -13882,7 +13882,7 @@
       </c>
       <c r="H269" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I269" s="4" t="inlineStr">
@@ -13932,7 +13932,7 @@
       </c>
       <c r="H270" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I270" s="4" t="inlineStr">
@@ -13982,7 +13982,7 @@
       </c>
       <c r="H271" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I271" s="4" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="H272" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I272" s="4" t="inlineStr">
@@ -14082,7 +14082,7 @@
       </c>
       <c r="H273" s="4" t="inlineStr">
         <is>
-          <t>affil</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="I273" s="4" t="inlineStr">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>⭐ 双满足 = 机构署名 + InnoHK致谢 (103 篇) | 黄色高亮 = 双满足 + 近30天发表 (1 篇) | 灰色 = 单通道</t>
+          <t>⭐ Dual-Channel = COCHE affiliation + InnoHK/ITC acknowledgement (103 papers) | Gold highlight = Dual-Channel + published past 30 days (1 papers) | Grey text = single-channel</t>
         </is>
       </c>
     </row>

</xml_diff>